<commit_message>
chore(pel): pulizia progetto e aggiornamento testbook PEL
Pulizia:
- Aggiunge pytest_pel/pytest_pel/ a .gitignore (cartella nidificata
  stray, stesso problema gia' noto per pytest_playwright).
- Rimossi 26 screenshot di debug obsoleti dalla root (gia' gitignorati,
  solo pulizia disco locale).

Testbook (suite_test_pel.xlsx):
- Aggiunti i fogli Messaggi (25 test), Contatti (10), Archivio (2),
  Impostazioni (7) con lo stesso stile delle sezioni esistenti.
- Rinominato il foglio "Impostazioni" preesistente (2 test S1/S2 sul
  calendario) in "Impostazioni Calendario" per evitare la collisione
  di nome con il nuovo modulo Impostazioni generale.
- Aggiornati Suite Completa (ID 18-61) e Indice (nuovo totale: 61
  casi di test) di conseguenza.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/suite_test_pel.xlsx
+++ b/suite_test_pel.xlsx
@@ -10,8 +10,12 @@
     <sheet name="Indice" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Suite Completa" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Login" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Calendario" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Impostazioni" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Messaggi" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Calendario" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Contatti" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Impostazioni" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Archivio" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Impostazioni Calendario" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -159,7 +163,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -216,8 +220,32 @@
         <fgColor rgb="001D5F5F"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0E4D6"/>
+        <bgColor rgb="00F0E4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4D6F0"/>
+        <bgColor rgb="00E4D6F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6F0DC"/>
+        <bgColor rgb="00D6F0DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0D6E0"/>
+        <bgColor rgb="00F0D6E0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -253,11 +281,44 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -466,6 +527,41 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -832,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -920,7 +1016,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Impostazioni</t>
+          <t>Impostazioni Calendario</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
@@ -933,21 +1029,94 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="72" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C8" s="71" t="n">
+        <v>25</v>
+      </c>
+      <c r="D8" s="71" t="inlineStr">
+        <is>
+          <t>Test sulla gestione dei messaggi PEL: invio, ricezione, risposta, allegati, cartelle, etichette, filtri, modelli e funzioni avanzate. Esclusi 2 test su ricevute RA/RD (ambiente di test non su dominio PEC certificato).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="73" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>Contatti</t>
+        </is>
+      </c>
+      <c r="C9" s="73" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="73" t="inlineStr">
+        <is>
+          <t>Test sulla rubrica contatti PEL: aggiunta, modifica, eliminazione, ricerca, gruppi, preferiti, import/export CSV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="75" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>Archivio</t>
+        </is>
+      </c>
+      <c r="C10" s="75" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="75" t="inlineStr">
+        <is>
+          <t>Test sulla funzionalità Archivio: configurazione delle regole di archiviazione e verifica dell'archiviazione effettiva. Fa skip automatico sulle caselle PEL dove la feature non è disponibile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="77" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="78" t="inlineStr">
+        <is>
+          <t>Impostazioni</t>
+        </is>
+      </c>
+      <c r="C11" s="77" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" s="77" t="inlineStr">
+        <is>
+          <t>Test sulle impostazioni generali della casella PEL: firme, riquadro di lettura, regole messaggi, risposta automatica, posta indesiderata, cestino e storico accessi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>TOTALE CASI DI TEST</t>
         </is>
       </c>
-      <c r="C8" s="13" t="n">
-        <v>17</v>
-      </c>
-      <c r="D8" s="14" t="n"/>
+      <c r="B12" s="79" t="n"/>
+      <c r="C12" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="D12" s="80" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A8:B8"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -959,7 +1128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1670,7 +1839,7 @@
       </c>
       <c r="B18" s="36" t="inlineStr">
         <is>
-          <t>Impostazioni</t>
+          <t>Impostazioni Calendario</t>
         </is>
       </c>
       <c r="C18" s="37" t="inlineStr">
@@ -1716,7 +1885,7 @@
       </c>
       <c r="B19" s="42" t="inlineStr">
         <is>
-          <t>Impostazioni</t>
+          <t>Impostazioni Calendario</t>
         </is>
       </c>
       <c r="C19" s="24" t="inlineStr">
@@ -1751,6 +1920,1840 @@
       <c r="G19" s="28" t="inlineStr">
         <is>
           <t>Se la selezione della vista 'Mese' è riuscita: il calendario si apre in vista Mese. Se il combobox usa shadow DOM non interagibile: la pagina impostazioni è accessibile (PASS con fallback).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="83" customHeight="1">
+      <c r="A20" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_01.py</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggio_con_allegato</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t>Verifica l'invio di un messaggio PEL con allegato e la sua corretta visualizzazione.</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire l'indirizzo del destinatario principale.
+4. Inserire oggetto e corpo del messaggio.
+5. Allegare un file PDF tramite il pulsante allegati.
+6. Inviare il messaggio.
+7. Attendere la ricezione nella cartella In arrivo.
+8. Aprire il messaggio ricevuto.
+9. Scattare screenshot.
+10. Verificare la presenza dell'allegato nel messaggio (assert).</t>
+        </is>
+      </c>
+      <c r="G20" s="23" t="inlineStr">
+        <is>
+          <t>Il messaggio è presente in In arrivo. L'allegato è visibile all'interno del messaggio ricevuto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="72" customHeight="1">
+      <c r="A21" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggi_02.py</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggio_inoltrato</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>Verifica l'inoltro di un messaggio PEL ricevuto.</t>
+        </is>
+      </c>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare un messaggio a se stessi con oggetto univoco.
+3. Attendere la ricezione del messaggio.
+4. Aprire il messaggio ricevuto.
+5. Cliccare il pulsante 'Inoltra'.
+6. Inserire il destinatario dell'inoltro.
+7. Inviare il messaggio inoltrato.
+8. Scattare screenshot.
+9. Verificare la comparsa del toast di conferma (assert).</t>
+        </is>
+      </c>
+      <c r="G21" s="17" t="inlineStr">
+        <is>
+          <t>Il messaggio inoltrato è inviato correttamente. Il toast di conferma è visibile. L'oggetto contiene il prefisso di inoltro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="61" customHeight="1">
+      <c r="A22" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_03.py</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggio_in_bozza</t>
+        </is>
+      </c>
+      <c r="E22" s="23" t="inlineStr">
+        <is>
+          <t>Verifica il salvataggio di un messaggio come bozza e il successivo invio.</t>
+        </is>
+      </c>
+      <c r="F22" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire destinatario, oggetto e corpo.
+4. Cliccare 'Salva bozza' (o chiudere la finestra senza inviare).
+5. Navigare nella cartella Bozze.
+6. Verificare che la bozza sia presente.
+7. Aprire la bozza e inviarla.
+8. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="G22" s="23" t="inlineStr">
+        <is>
+          <t>La bozza è visibile nella cartella Bozze. Dopo l'invio, la bozza non è più presente nella cartella Bozze.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="55.6" customHeight="1">
+      <c r="A23" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggi_04.py</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggio_importato</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>Verifica l'importazione di messaggi da file nella casella PEL.</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Aprire il menu di importazione messaggi.
+3. Selezionare il file da importare.
+4. Avviare il processo di importazione.
+5. Attendere il completamento dell'importazione.
+6. Scattare screenshot.
+7. Verificare il messaggio di conferma (assert).</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="inlineStr">
+        <is>
+          <t>Il processo di importazione si completa senza errori. Viene mostrato un messaggio di successo o conferma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="68.59999999999999" customHeight="1">
+      <c r="A24" s="23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_05.py</t>
+        </is>
+      </c>
+      <c r="D24" s="23" t="inlineStr">
+        <is>
+          <t>test_cartella</t>
+        </is>
+      </c>
+      <c r="E24" s="23" t="inlineStr">
+        <is>
+          <t>Verifica la creazione, la modifica e l'eliminazione di una cartella personalizzata.</t>
+        </is>
+      </c>
+      <c r="F24" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare una nuova cartella con nome univoco.
+3. Verificare il toast di conferma della creazione.
+4. Rinominare la cartella con un nuovo nome.
+5. Verificare il toast di conferma della modifica.
+6. Eliminare la cartella.
+7. Scattare screenshot.
+8. Verificare il toast di conferma dell'eliminazione (assert).</t>
+        </is>
+      </c>
+      <c r="G24" s="23" t="inlineStr">
+        <is>
+          <t>La cartella è creata, rinominata ed eliminata con successo. Per ogni operazione compare un toast di conferma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="72.2" customHeight="1">
+      <c r="A25" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggi_06.py</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>test_ripristino_messaggi</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>Verifica il ripristino di messaggi dal cestino alla cartella In arrivo.</t>
+        </is>
+      </c>
+      <c r="F25" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Spostare un messaggio nel cestino.
+3. Navigare nella cartella Cestino.
+4. Selezionare il/i messaggio/i da ripristinare.
+5. Cliccare 'Ripristina' o 'Sposta in In arrivo'.
+6. Verificare che i messaggi non siano più nel cestino.
+7. Scattare screenshot.
+8. Navigare in In arrivo e verificare la presenza dei messaggi (assert).</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="inlineStr">
+        <is>
+          <t>I messaggi ripristinati non sono più nel cestino e sono visibili nella cartella In arrivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="68.59999999999999" customHeight="1">
+      <c r="A26" s="23" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_07.py</t>
+        </is>
+      </c>
+      <c r="D26" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_preferiti_pinnati</t>
+        </is>
+      </c>
+      <c r="E26" s="23" t="inlineStr">
+        <is>
+          <t>Verifica l'aggiunta di messaggi ai preferiti e la funzione 'Pinna messaggio'.</t>
+        </is>
+      </c>
+      <c r="F26" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Selezionare un messaggio dall'In arrivo.
+3. Aggiungere il messaggio ai preferiti (stella).
+4. Verificare che il messaggio compaia nella cartella Preferiti/Speciali.
+5. Selezionare un messaggio e cliccare 'Pinna messaggio'.
+6. Scattare screenshot.
+7. Verificare la presenza del messaggio pinnato (assert).</t>
+        </is>
+      </c>
+      <c r="G26" s="23" t="inlineStr">
+        <is>
+          <t>Il messaggio è aggiunto ai preferiti e compare nella sezione Preferiti. Il messaggio pinnato è visibile in cima alla lista.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="70.40000000000001" customHeight="1">
+      <c r="A27" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggi_08.py</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>test_etichetta</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>Verifica la creazione di un'etichetta, la sua applicazione ai messaggi e l'eliminazione.</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Aprire le impostazioni etichette.
+3. Creare una nuova etichetta con nome univoco e colore.
+4. Tornare in In arrivo e selezionare un messaggio.
+5. Applicare l'etichetta appena creata al messaggio.
+6. Verificare che l'etichetta sia visibile sul messaggio.
+7. Scattare screenshot.
+8. Eliminare l'etichetta (cleanup).</t>
+        </is>
+      </c>
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>L'etichetta è creata e applicata con successo al messaggio. Dopo l'eliminazione dell'etichetta, essa non è più visibile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="68.2" customHeight="1">
+      <c r="A28" s="23" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_09.py</t>
+        </is>
+      </c>
+      <c r="D28" s="23" t="inlineStr">
+        <is>
+          <t>test_segna_come_letto_da_leggere</t>
+        </is>
+      </c>
+      <c r="E28" s="23" t="inlineStr">
+        <is>
+          <t>Verifica le funzioni 'Segna come letto' e 'Segna come da leggere' sui messaggi.</t>
+        </is>
+      </c>
+      <c r="F28" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Selezionare un messaggio non letto dall'In arrivo.
+3. Cliccare 'Segna come letto'.
+4. Verificare che il messaggio non sia più in grassetto (letto).
+5. Cliccare 'Segna come da leggere' sullo stesso messaggio.
+6. Scattare screenshot.
+7. Verificare che il messaggio torni in grassetto (non letto, assert).</t>
+        </is>
+      </c>
+      <c r="G28" s="23" t="inlineStr">
+        <is>
+          <t>I pulsanti 'Segna come letto' e 'Segna come da leggere' sono visibili e funzionanti. Lo stato del messaggio cambia correttamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="70" customHeight="1">
+      <c r="A29" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggi_10.py</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggio_alta_priorita</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>Verifica l'invio e la ricezione di un messaggio con priorità alta.</t>
+        </is>
+      </c>
+      <c r="F29" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire destinatario, oggetto e corpo.
+4. Impostare la priorità del messaggio su 'Alta'.
+5. Inviare il messaggio.
+6. Attendere la ricezione in In arrivo.
+7. Aprire il messaggio ricevuto.
+8. Scattare screenshot.
+9. Verificare la presenza dell'indicatore di alta priorità (assert).</t>
+        </is>
+      </c>
+      <c r="G29" s="17" t="inlineStr">
+        <is>
+          <t>Il messaggio è ricevuto con l'indicatore di alta priorità visibile (simbolo '!' o equivalente).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="61.4" customHeight="1">
+      <c r="A30" s="23" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_11.py</t>
+        </is>
+      </c>
+      <c r="D30" s="23" t="inlineStr">
+        <is>
+          <t>test_risposta_messaggio</t>
+        </is>
+      </c>
+      <c r="E30" s="23" t="inlineStr">
+        <is>
+          <t>Verifica la risposta a un messaggio PEL ricevuto.</t>
+        </is>
+      </c>
+      <c r="F30" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare un messaggio a se stessi.
+3. Attendere la ricezione del messaggio.
+4. Aprire il messaggio ricevuto.
+5. Cliccare il pulsante 'Rispondi'.
+6. Verificare che la finestra di risposta sia aperta con 'Re:' nell'oggetto.
+7. Inviare la risposta.
+8. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="G30" s="23" t="inlineStr">
+        <is>
+          <t>La finestra di risposta si apre correttamente. L'oggetto contiene il prefisso 'Re:'. La risposta viene inviata con successo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="52" customHeight="1">
+      <c r="A31" s="17" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggi_12.py</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>test_invio_messaggio_semplice</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>Verifica l'invio di un messaggio PEL semplice senza allegati.</t>
+        </is>
+      </c>
+      <c r="F31" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire l'indirizzo del destinatario.
+4. Inserire oggetto e corpo del messaggio.
+5. Cliccare 'Invia'.
+6. Scattare screenshot.
+7. Verificare la comparsa del toast di conferma invio (assert).</t>
+        </is>
+      </c>
+      <c r="G31" s="17" t="inlineStr">
+        <is>
+          <t>Il messaggio è inviato con successo. Appare un toast di conferma dell'invio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="77.2" customHeight="1">
+      <c r="A32" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C32" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_13.py</t>
+        </is>
+      </c>
+      <c r="D32" s="23" t="inlineStr">
+        <is>
+          <t>test_risposta_a_tutti</t>
+        </is>
+      </c>
+      <c r="E32" s="23" t="inlineStr">
+        <is>
+          <t>Verifica la funzione 'Rispondi a tutti' su un messaggio ricevuto.</t>
+        </is>
+      </c>
+      <c r="F32" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare un messaggio a se stessi.
+3. Attendere la ricezione del messaggio.
+4. Aprire il messaggio ricevuto.
+5. Cliccare il pulsante 'Rispondi a tutti'.
+6. Verificare che la finestra di risposta sia aperta con 'Re:' nell'oggetto.
+7. Verificare che tutti i destinatari originali siano inclusi.
+8. Inviare la risposta a tutti.
+9. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="G32" s="23" t="inlineStr">
+        <is>
+          <t>La finestra di risposta si apre con l'oggetto 'Re: ...' e tutti i destinatari originali inclusi. La risposta viene inviata con successo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="63.8" customHeight="1">
+      <c r="A33" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggi_14.py</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>test_elimina_messaggio</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>Verifica l'eliminazione di un messaggio e la sua presenza nel cestino.</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare un messaggio a se stessi con oggetto univoco.
+3. Attendere la ricezione del messaggio.
+4. Selezionare il messaggio e cliccare 'Elimina'.
+5. Navigare nella cartella Cestino.
+6. Scattare screenshot.
+7. Verificare che il messaggio eliminato sia presente nel cestino (assert).</t>
+        </is>
+      </c>
+      <c r="G33" s="17" t="inlineStr">
+        <is>
+          <t>Il messaggio eliminato non è più in In arrivo ma è visibile nella cartella Cestino.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="86.40000000000001" customHeight="1">
+      <c r="A34" s="23" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_15.py</t>
+        </is>
+      </c>
+      <c r="D34" s="23" t="inlineStr">
+        <is>
+          <t>test_sposta_messaggio_in_cartella</t>
+        </is>
+      </c>
+      <c r="E34" s="23" t="inlineStr">
+        <is>
+          <t>Verifica lo spostamento di un messaggio in una cartella personalizzata.</t>
+        </is>
+      </c>
+      <c r="F34" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare una nuova cartella con nome univoco.
+3. Inviare un messaggio a se stessi.
+4. Attendere la ricezione del messaggio.
+5. Selezionare il messaggio e cliccare 'Sposta in...'.
+6. Selezionare la cartella di destinazione.
+7. Verificare che il messaggio non sia più in In arrivo.
+8. Scattare screenshot.
+9. Navigare nella cartella di destinazione e verificare la presenza del messaggio (assert).</t>
+        </is>
+      </c>
+      <c r="G34" s="23" t="inlineStr">
+        <is>
+          <t>Il messaggio è spostato correttamente nella cartella di destinazione e non è più visibile in In arrivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="76.8" customHeight="1">
+      <c r="A35" s="17" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggi_16.py</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>test_copia_messaggio_in_cartella</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>Verifica la copia di un messaggio in una cartella personalizzata.</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare una nuova cartella con nome univoco.
+3. Aprire un messaggio esistente in In arrivo.
+4. Selezionare 'Copia in...' dal menu azioni.
+5. Selezionare la cartella di destinazione.
+6. Verificare che il messaggio originale sia ancora in In arrivo.
+7. Scattare screenshot.
+8. Navigare nella cartella di destinazione e verificare la copia (assert).</t>
+        </is>
+      </c>
+      <c r="G35" s="17" t="inlineStr">
+        <is>
+          <t>Il messaggio è copiato nella cartella di destinazione. Il messaggio originale rimane in In arrivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="60.6" customHeight="1">
+      <c r="A36" s="23" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C36" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_17.py</t>
+        </is>
+      </c>
+      <c r="D36" s="23" t="inlineStr">
+        <is>
+          <t>test_ricerca_messaggi</t>
+        </is>
+      </c>
+      <c r="E36" s="23" t="inlineStr">
+        <is>
+          <t>Verifica la funzione di ricerca messaggi nella casella PEL.</t>
+        </is>
+      </c>
+      <c r="F36" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare un messaggio a se stessi con oggetto univoco.
+3. Attendere la ricezione del messaggio.
+4. Inserire il testo univoco nella barra di ricerca.
+5. Avviare la ricerca.
+6. Scattare screenshot.
+7. Verificare che il messaggio cercato appaia nei risultati (assert).</t>
+        </is>
+      </c>
+      <c r="G36" s="23" t="inlineStr">
+        <is>
+          <t>Il messaggio con l'oggetto univoco è trovato e visibile nei risultati di ricerca.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="63.2" customHeight="1">
+      <c r="A37" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggi_18.py</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>test_filtri_inbox</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>Verifica la presenza e il funzionamento del filtro messaggi (Tutti/Letti/Da leggere) nella lista In arrivo.</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Attendere che i messaggi siano visibili in In arrivo.
+3. Individuare il filtro 'Letti' tra i tab aru-chip in alto alla lista.
+4. Cliccare il filtro 'Letti'.
+5. Scattare screenshot.
+6. Verificare che l'URL rifletta il quick-filter applicato (parametro mail_quickFilter, assert).</t>
+        </is>
+      </c>
+      <c r="G37" s="17" t="inlineStr">
+        <is>
+          <t>Il filtro 'Letti' è visibile e cliccabile. Dopo il click l'URL contiene il parametro 'mail_quickFilter', confermando che il filtro è stato applicato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="57.8" customHeight="1">
+      <c r="A38" s="23" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_19.py</t>
+        </is>
+      </c>
+      <c r="D38" s="23" t="inlineStr">
+        <is>
+          <t>test_invio_messaggio_con_cc</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="inlineStr">
+        <is>
+          <t>Verifica l'invio di un messaggio PEL con destinatario in copia (CC).</t>
+        </is>
+      </c>
+      <c r="F38" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire l'indirizzo del destinatario principale.
+4. Aggiungere un destinatario in CC.
+5. Inserire oggetto e corpo del messaggio.
+6. Cliccare 'Invia'.
+7. Scattare screenshot.
+8. Verificare la conferma di invio (assert).</t>
+        </is>
+      </c>
+      <c r="G38" s="23" t="inlineStr">
+        <is>
+          <t>Il messaggio è inviato con successo con entrambi i destinatari (To e CC). Appare il toast di conferma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="84.40000000000001" customHeight="1">
+      <c r="A39" s="17" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggi_20.py</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>test_scarica_allegato_ricevuto</t>
+        </is>
+      </c>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>Verifica il download di un allegato da un messaggio PEL ricevuto.</t>
+        </is>
+      </c>
+      <c r="F39" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare a se stessi un messaggio con allegato PDF.
+3. Attendere la ricezione del messaggio.
+4. Aprire il messaggio ricevuto.
+5. Cliccare sul pulsante di download dell'allegato.
+6. Gestire il download tramite Playwright expect_download.
+7. Salvare il file nella cartella test-results.
+8. Scattare screenshot.
+9. Verificare che il file scaricato esista e abbia dimensione &gt; 0 (assert).</t>
+        </is>
+      </c>
+      <c r="G39" s="17" t="inlineStr">
+        <is>
+          <t>Il file allegato viene scaricato correttamente. Il file esiste nella directory di destinazione e ha dimensione maggiore di 0 byte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="63.4" customHeight="1">
+      <c r="A40" s="23" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_21.py</t>
+        </is>
+      </c>
+      <c r="D40" s="23" t="inlineStr">
+        <is>
+          <t>test_salva_e_usa_modello</t>
+        </is>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>Verifica il salvataggio di un messaggio come modello e il suo successivo utilizzo.</t>
+        </is>
+      </c>
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire oggetto e corpo del messaggio modello.
+4. Salvare come modello invece di inviare.
+5. Navigare nella cartella Modelli.
+6. Verificare che il modello sia presente.
+7. Aprire il modello e inviarlo come nuovo messaggio.
+8. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="G40" s="23" t="inlineStr">
+        <is>
+          <t>Il modello è salvato e visibile nella cartella Modelli. Può essere aperto e utilizzato per inviare un nuovo messaggio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="60" customHeight="1">
+      <c r="A41" s="17" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggi_22.py</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>test_verifica_cartella_inviati</t>
+        </is>
+      </c>
+      <c r="E41" s="17" t="inlineStr">
+        <is>
+          <t>Verifica che i messaggi inviati siano presenti nella cartella Inviati.</t>
+        </is>
+      </c>
+      <c r="F41" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare un messaggio con oggetto univoco.
+3. Attendere la conferma di invio.
+4. Navigare nella cartella Inviati.
+5. Cercare il messaggio con l'oggetto univoco.
+6. Scattare screenshot.
+7. Verificare che il messaggio sia presente con il corretto oggetto (assert).</t>
+        </is>
+      </c>
+      <c r="G41" s="17" t="inlineStr">
+        <is>
+          <t>Il messaggio inviato è visibile nella cartella Inviati con l'oggetto corretto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="67.59999999999999" customHeight="1">
+      <c r="A42" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C42" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_25.py</t>
+        </is>
+      </c>
+      <c r="D42" s="23" t="inlineStr">
+        <is>
+          <t>test_invio_allegati_multipli</t>
+        </is>
+      </c>
+      <c r="E42" s="23" t="inlineStr">
+        <is>
+          <t>Verifica l'invio di un messaggio con allegati multipli.</t>
+        </is>
+      </c>
+      <c r="F42" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire destinatario, oggetto e corpo.
+4. Cliccare il pulsante allegati e selezionare il primo file.
+5. Aggiungere un secondo allegato.
+6. Verificare che almeno 2 allegati siano visibili nella finestra di composizione.
+7. Inviare il messaggio.
+8. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="G42" s="23" t="inlineStr">
+        <is>
+          <t>Almeno 2 allegati sono visibili nella finestra di composizione prima dell'invio. Il messaggio viene inviato con successo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="83.40000000000001" customHeight="1">
+      <c r="A43" s="17" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="17" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>test_messaggi_26.py</t>
+        </is>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>test_selezione_multipla_batch</t>
+        </is>
+      </c>
+      <c r="E43" s="17" t="inlineStr">
+        <is>
+          <t>Verifica la selezione multipla di messaggi e la comparsa della toolbar azioni batch.</t>
+        </is>
+      </c>
+      <c r="F43" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare 2 messaggi a se stessi con oggetti univoci.
+3. Attendere la ricezione di entrambi in In arrivo.
+4. Passare il mouse sulla prima riga messaggio per rivelare il checkbox.
+5. Selezionare il checkbox della prima riga.
+6. Passare il mouse sulla seconda riga e selezionare il suo checkbox.
+7. Scattare screenshot.
+8. Verificare la comparsa della toolbar azioni batch (assert).</t>
+        </is>
+      </c>
+      <c r="G43" s="17" t="inlineStr">
+        <is>
+          <t>Dopo la selezione di almeno 2 messaggi, la toolbar delle azioni batch è visibile con i relativi pulsanti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="69.8" customHeight="1">
+      <c r="A44" s="23" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="23" t="inlineStr">
+        <is>
+          <t>Messaggi</t>
+        </is>
+      </c>
+      <c r="C44" s="23" t="inlineStr">
+        <is>
+          <t>test_messaggi_27.py</t>
+        </is>
+      </c>
+      <c r="D44" s="23" t="inlineStr">
+        <is>
+          <t>test_anomalia_invio_non_pec</t>
+        </is>
+      </c>
+      <c r="E44" s="23" t="inlineStr">
+        <is>
+          <t>Verifica che l'invio a un indirizzo non-PEC generi una notifica di anomalia.</t>
+        </is>
+      </c>
+      <c r="F44" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire un indirizzo email non-PEC come destinatario.
+4. Inserire oggetto e corpo del messaggio.
+5. Inviare il messaggio.
+6. Attendere la ricezione della notifica di anomalia.
+7. Scattare screenshot.
+8. Verificare la presenza della notifica nell'inbox o come avviso UI (assert).</t>
+        </is>
+      </c>
+      <c r="G44" s="23" t="inlineStr">
+        <is>
+          <t>Viene generata e ricevuta una notifica di anomalia per l'invio a un indirizzo non-PEC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="56.8" customHeight="1">
+      <c r="A45" s="17" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" s="17" t="inlineStr">
+        <is>
+          <t>Contatti</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="inlineStr">
+        <is>
+          <t>test_contatti_01.py</t>
+        </is>
+      </c>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>test_aggiungere_nuovo_contatto</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="inlineStr">
+        <is>
+          <t>Verifica la creazione di un nuovo contatto nella rubrica della casella PEL.</t>
+        </is>
+      </c>
+      <c r="F45" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare nella sezione Contatti.
+3. Cliccare 'Nuovo contatto'.
+4. Inserire nome, cognome e indirizzo email.
+5. Salvare il contatto.
+6. Verificare la presenza del contatto nella rubrica.
+7. Scattare screenshot.
+8. Eliminare il contatto (cleanup).</t>
+        </is>
+      </c>
+      <c r="G45" s="17" t="inlineStr">
+        <is>
+          <t>Il contatto è creato e visibile nella rubrica con nome, cognome e email corretti. Può essere eliminato correttamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="66.59999999999999" customHeight="1">
+      <c r="A46" s="23" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" s="23" t="inlineStr">
+        <is>
+          <t>Contatti</t>
+        </is>
+      </c>
+      <c r="C46" s="23" t="inlineStr">
+        <is>
+          <t>test_contatti_02.py</t>
+        </is>
+      </c>
+      <c r="D46" s="23" t="inlineStr">
+        <is>
+          <t>test_aggiungere_nuovo_gruppo</t>
+        </is>
+      </c>
+      <c r="E46" s="23" t="inlineStr">
+        <is>
+          <t>Verifica la creazione di un gruppo contatti e l'aggiunta di contatti al gruppo.</t>
+        </is>
+      </c>
+      <c r="F46" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare nella sezione Contatti.
+3. Cliccare 'Nuovo gruppo'.
+4. Inserire il nome del gruppo.
+5. Salvare il gruppo.
+6. Aggiungere uno o più contatti al gruppo.
+7. Verificare che il gruppo sia visibile nella sidebar.
+8. Scattare screenshot.
+9. Verificare che i contatti siano nel gruppo (assert).</t>
+        </is>
+      </c>
+      <c r="G46" s="23" t="inlineStr">
+        <is>
+          <t>Il gruppo è creato e visibile nella sidebar. I contatti aggiunti sono visibili nel gruppo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="68" customHeight="1">
+      <c r="A47" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" s="17" t="inlineStr">
+        <is>
+          <t>Contatti</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>test_contatti_03.py</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>test_esporta_contatti</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>Verifica l'esportazione della rubrica contatti in formato CSV.</t>
+        </is>
+      </c>
+      <c r="F47" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare nella sezione Contatti.
+3. Aprire il menu Opzioni della rubrica.
+4. Selezionare 'Esporta rubrica'.
+5. Gestire il download del file tramite Playwright expect_download.
+6. Verificare che il file CSV sia scaricato.
+7. Scattare screenshot.
+8. Verificare che il file abbia dimensione &gt; 0 (assert).</t>
+        </is>
+      </c>
+      <c r="G47" s="17" t="inlineStr">
+        <is>
+          <t>Il file CSV della rubrica è scaricato correttamente con dimensione maggiore di 0 byte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="58.4" customHeight="1">
+      <c r="A48" s="23" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" s="23" t="inlineStr">
+        <is>
+          <t>Contatti</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="inlineStr">
+        <is>
+          <t>test_contatti_04.py</t>
+        </is>
+      </c>
+      <c r="D48" s="23" t="inlineStr">
+        <is>
+          <t>test_importa_contatti</t>
+        </is>
+      </c>
+      <c r="E48" s="23" t="inlineStr">
+        <is>
+          <t>Verifica l'importazione di contatti da un file CSV nella rubrica PEL.</t>
+        </is>
+      </c>
+      <c r="F48" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare nella sezione Contatti.
+3. Cliccare 'Importa'.
+4. Selezionare il file CSV di test tramite il file picker.
+5. Confermare l'importazione.
+6. Verificare il messaggio di successo.
+7. Scattare screenshot.
+8. Eliminare i contatti importati (cleanup).</t>
+        </is>
+      </c>
+      <c r="G48" s="23" t="inlineStr">
+        <is>
+          <t>I contatti del file CSV sono importati con successo nella rubrica. Il messaggio di conferma è visibile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="70" customHeight="1">
+      <c r="A49" s="17" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" s="17" t="inlineStr">
+        <is>
+          <t>Contatti</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>test_contatti_05.py</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>test_modifica_contatto</t>
+        </is>
+      </c>
+      <c r="E49" s="17" t="inlineStr">
+        <is>
+          <t>Verifica la modifica dei dati di un contatto esistente nella rubrica.</t>
+        </is>
+      </c>
+      <c r="F49" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare un contatto da modificare.
+3. Cercare il contatto.
+4. Aprirlo e cliccare 'Modifica'.
+5. Cambiare il cognome con un valore nuovo univoco.
+6. Salvare le modifiche.
+7. Cercare il contatto con il nuovo cognome.
+8. Scattare screenshot.
+9. Verificare che il contatto sia trovato con i dati aggiornati (assert).</t>
+        </is>
+      </c>
+      <c r="G49" s="17" t="inlineStr">
+        <is>
+          <t>Il contatto è modificato correttamente. La ricerca con il nuovo cognome restituisce il contatto aggiornato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="57" customHeight="1">
+      <c r="A50" s="23" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" s="23" t="inlineStr">
+        <is>
+          <t>Contatti</t>
+        </is>
+      </c>
+      <c r="C50" s="23" t="inlineStr">
+        <is>
+          <t>test_contatti_06.py</t>
+        </is>
+      </c>
+      <c r="D50" s="23" t="inlineStr">
+        <is>
+          <t>test_elimina_contatto</t>
+        </is>
+      </c>
+      <c r="E50" s="23" t="inlineStr">
+        <is>
+          <t>Verifica l'eliminazione di un contatto dalla rubrica.</t>
+        </is>
+      </c>
+      <c r="F50" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare un contatto di test con nome univoco.
+3. Selezionare il contatto.
+4. Cliccare 'Elimina'.
+5. Confermare l'eliminazione.
+6. Cercare il contatto eliminato.
+7. Scattare screenshot.
+8. Verificare che non sia più presente nella rubrica (assert).</t>
+        </is>
+      </c>
+      <c r="G50" s="23" t="inlineStr">
+        <is>
+          <t>Il contatto eliminato non è più presente nella rubrica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="53.4" customHeight="1">
+      <c r="A51" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" s="17" t="inlineStr">
+        <is>
+          <t>Contatti</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="inlineStr">
+        <is>
+          <t>test_contatti_07.py</t>
+        </is>
+      </c>
+      <c r="D51" s="17" t="inlineStr">
+        <is>
+          <t>test_ricerca_contatto</t>
+        </is>
+      </c>
+      <c r="E51" s="17" t="inlineStr">
+        <is>
+          <t>Verifica la ricerca di un contatto nella rubrica tramite la barra di ricerca.</t>
+        </is>
+      </c>
+      <c r="F51" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare un contatto con nome univoco.
+3. Inserire il nome univoco nella barra di ricerca.
+4. Avviare la ricerca.
+5. Verificare che il contatto cercato sia nei risultati.
+6. Scattare screenshot.
+7. Eliminare il contatto (cleanup).</t>
+        </is>
+      </c>
+      <c r="G51" s="17" t="inlineStr">
+        <is>
+          <t>Il contatto con il nome univoco è trovato e visibile nei risultati di ricerca della rubrica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="57.4" customHeight="1">
+      <c r="A52" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" s="23" t="inlineStr">
+        <is>
+          <t>Contatti</t>
+        </is>
+      </c>
+      <c r="C52" s="23" t="inlineStr">
+        <is>
+          <t>test_contatti_08.py</t>
+        </is>
+      </c>
+      <c r="D52" s="23" t="inlineStr">
+        <is>
+          <t>test_contatto_preferito</t>
+        </is>
+      </c>
+      <c r="E52" s="23" t="inlineStr">
+        <is>
+          <t>Verifica l'aggiunta di un contatto ai preferiti e la sua visualizzazione nella sezione Preferiti.</t>
+        </is>
+      </c>
+      <c r="F52" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Selezionare un contatto dalla rubrica.
+3. Cliccare il pulsante stella (preferito).
+4. Navigare nella sezione 'Contatti preferiti' nella sidebar.
+5. Verificare che il contatto sia presente.
+6. Scattare screenshot.
+7. Eliminare il contatto (cleanup).</t>
+        </is>
+      </c>
+      <c r="G52" s="23" t="inlineStr">
+        <is>
+          <t>Il contatto aggiunto ai preferiti è visibile nella sezione Contatti preferiti nella sidebar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="62.6" customHeight="1">
+      <c r="A53" s="17" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" s="17" t="inlineStr">
+        <is>
+          <t>Contatti</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>test_contatti_09.py</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>test_scrivi_email_da_contatto</t>
+        </is>
+      </c>
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>Verifica l'apertura della finestra di composizione email direttamente da un contatto.</t>
+        </is>
+      </c>
+      <c r="F53" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare un contatto con email.
+3. Cercarlo nella rubrica.
+4. Cliccare il pulsante azione per scrivere email dal contatto.
+5. Verificare che la finestra di composizione si apra.
+6. Scattare screenshot.
+7. Chiudere il composer senza inviare.
+8. Eliminare il contatto (cleanup).</t>
+        </is>
+      </c>
+      <c r="G53" s="17" t="inlineStr">
+        <is>
+          <t>La finestra di composizione si apre correttamente a partire dal contatto selezionato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="57.6" customHeight="1">
+      <c r="A54" s="23" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" s="23" t="inlineStr">
+        <is>
+          <t>Contatti</t>
+        </is>
+      </c>
+      <c r="C54" s="23" t="inlineStr">
+        <is>
+          <t>test_contatti_10.py</t>
+        </is>
+      </c>
+      <c r="D54" s="23" t="inlineStr">
+        <is>
+          <t>test_elimina_gruppo</t>
+        </is>
+      </c>
+      <c r="E54" s="23" t="inlineStr">
+        <is>
+          <t>Verifica la creazione e l'eliminazione di un gruppo contatti.</t>
+        </is>
+      </c>
+      <c r="F54" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare un nuovo gruppo con nome univoco.
+3. Verificare la presenza del gruppo nella sidebar.
+4. Tasto destro sul gruppo ed Elimina.
+5. Confermare l'eliminazione.
+6. Scattare screenshot.
+7. Verificare che il gruppo non sia più nella sidebar (assert).</t>
+        </is>
+      </c>
+      <c r="G54" s="23" t="inlineStr">
+        <is>
+          <t>Il gruppo è eliminato correttamente e non è più visibile nella sidebar dei contatti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="112.8" customHeight="1">
+      <c r="A55" s="17" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" s="17" t="inlineStr">
+        <is>
+          <t>Archivio</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="inlineStr">
+        <is>
+          <t>test_archivio_01.py</t>
+        </is>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>test_configurazione_archivio</t>
+        </is>
+      </c>
+      <c r="E55" s="17" t="inlineStr">
+        <is>
+          <t>Verifica la pagina di configurazione archivio: struttura, radio button e checkbox opzioni. Skip se la feature non è disponibile sull'account.</t>
+        </is>
+      </c>
+      <c r="F55" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare direttamente a /new/settings/archive.
+3. Se l'h1 'Archivio' non è visibile entro 10s, skip (feature non disponibile).
+4. Verificare h1 'Archivio' e h2 'Configurazione Archivio'.
+5. Verificare almeno 2 radio button e le checkbox opzioni (RA, RD, PEC ricevute/inviate).
+6. Selezionare 'Scegli quali messaggi archiviare' e una checkbox.
+7. Salvare e verificare il toast di conferma.
+8. Ricaricare e verificare che la selezione sia mantenuta.
+9. Scattare screenshot.
+10. Cleanup: ripristinare 'Archivia tutti' e salvare.</t>
+        </is>
+      </c>
+      <c r="G55" s="17" t="inlineStr">
+        <is>
+          <t>La pagina di configurazione Archivio mostra la struttura attesa e il salvataggio persiste dopo reload, oppure il test fa skip pulito se la feature non è presente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="113.8" customHeight="1">
+      <c r="A56" s="23" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" s="23" t="inlineStr">
+        <is>
+          <t>Archivio</t>
+        </is>
+      </c>
+      <c r="C56" s="23" t="inlineStr">
+        <is>
+          <t>test_archivio_02.py</t>
+        </is>
+      </c>
+      <c r="D56" s="23" t="inlineStr">
+        <is>
+          <t>test_archivio_messaggio_inviato</t>
+        </is>
+      </c>
+      <c r="E56" s="23" t="inlineStr">
+        <is>
+          <t>Verifica che i messaggi inviati/ricevuti vengano archiviati secondo la configurazione impostata. Skip se la feature non è disponibile.</t>
+        </is>
+      </c>
+      <c r="F56" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare a /new/settings/archive; skip se la feature non è disponibile.
+3. Selezionare 'Archivia tutti i messaggi ricevuti o inviati' e salvare.
+4. Creare e inviare un messaggio PEL a se stessi con oggetto univoco.
+5. Attendere l'archiviazione (10s).
+6. Aprire la sezione Archivio tramite il menu waffle (9 punti) nell'header.
+7. Cercare il messaggio con l'oggetto univoco nella barra di ricerca dell'archivio.
+8. Scattare screenshot.
+9. Verificare che il messaggio sia presente (assert), con retry dopo 20s se non trovato subito.</t>
+        </is>
+      </c>
+      <c r="G56" s="23" t="inlineStr">
+        <is>
+          <t>Il messaggio inviato a se stessi compare nella sezione Archivio, oppure il test fa skip pulito se la feature non è presente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="51" customHeight="1">
+      <c r="A57" s="17" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" s="17" t="inlineStr">
+        <is>
+          <t>Impostazioni</t>
+        </is>
+      </c>
+      <c r="C57" s="17" t="inlineStr">
+        <is>
+          <t>test_impostazioni_01.py</t>
+        </is>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
+        <is>
+          <t>test_crea_firma</t>
+        </is>
+      </c>
+      <c r="E57" s="17" t="inlineStr">
+        <is>
+          <t>Verifica la creazione di una firma email nella sezione Impostazioni.</t>
+        </is>
+      </c>
+      <c r="F57" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare direttamente a /new/settings/messages-writing/signatures.
+3. Verificare l'header 'Firme'.
+4. Cliccare il pulsante di creazione firma.
+5. Inserire nome e testo della firma.
+6. Salvare.
+7. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="G57" s="17" t="inlineStr">
+        <is>
+          <t>La pagina Firme si carica correttamente e il form di creazione firma è compilabile e salvabile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="50" customHeight="1">
+      <c r="A58" s="23" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" s="23" t="inlineStr">
+        <is>
+          <t>Impostazioni</t>
+        </is>
+      </c>
+      <c r="C58" s="23" t="inlineStr">
+        <is>
+          <t>test_impostazioni_02.py</t>
+        </is>
+      </c>
+      <c r="D58" s="23" t="inlineStr">
+        <is>
+          <t>test_riquadro_di_lettura</t>
+        </is>
+      </c>
+      <c r="E58" s="23" t="inlineStr">
+        <is>
+          <t>Verifica la modifica della posizione del riquadro di lettura nei messaggi.</t>
+        </is>
+      </c>
+      <c r="F58" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare a Impostazioni &gt; Home.
+3. Verificare le opzioni 'A destra' e 'In basso'.
+4. Selezionare 'In basso'.
+5. Verificare il toast/cambio visivo.
+6. Scattare screenshot.
+7. Ripristinare 'A destra'.</t>
+        </is>
+      </c>
+      <c r="G58" s="23" t="inlineStr">
+        <is>
+          <t>Le opzioni del riquadro di lettura sono disponibili e selezionabili; la modifica viene applicata correttamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="60.8" customHeight="1">
+      <c r="A59" s="17" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" s="17" t="inlineStr">
+        <is>
+          <t>Impostazioni</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="inlineStr">
+        <is>
+          <t>test_impostazioni_03.py</t>
+        </is>
+      </c>
+      <c r="D59" s="17" t="inlineStr">
+        <is>
+          <t>test_regole_messaggi</t>
+        </is>
+      </c>
+      <c r="E59" s="17" t="inlineStr">
+        <is>
+          <t>Verifica l'accesso e la creazione di regole per i messaggi nelle Impostazioni.</t>
+        </is>
+      </c>
+      <c r="F59" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare direttamente a /new/settings/messages-writing/message-rules.
+3. Cliccare 'Nuova regola'.
+4. Verificare che il form (Nome regola, Condizioni, Azioni) sia visibile.
+5. Compilare il nome regola.
+6. Scattare screenshot.
+7. Eliminare la regola creata (cleanup).</t>
+        </is>
+      </c>
+      <c r="G59" s="17" t="inlineStr">
+        <is>
+          <t>La sezione Regole messaggi è accessibile e il form di creazione nuova regola si apre correttamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="50" customHeight="1">
+      <c r="A60" s="23" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" s="23" t="inlineStr">
+        <is>
+          <t>Impostazioni</t>
+        </is>
+      </c>
+      <c r="C60" s="23" t="inlineStr">
+        <is>
+          <t>test_impostazioni_04.py</t>
+        </is>
+      </c>
+      <c r="D60" s="23" t="inlineStr">
+        <is>
+          <t>test_risposta_automatica</t>
+        </is>
+      </c>
+      <c r="E60" s="23" t="inlineStr">
+        <is>
+          <t>Verifica l'accesso alla pagina 'Risposta automatica' nelle Impostazioni.</t>
+        </is>
+      </c>
+      <c r="F60" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare direttamente a /new/settings/messages-writing/automatic-reply.
+3. Verificare che l'h1 'Risposta automatica' sia visibile.
+4. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="G60" s="23" t="inlineStr">
+        <is>
+          <t>La pagina 'Risposta automatica' si carica correttamente con l'h1 atteso visibile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="62.2" customHeight="1">
+      <c r="A61" s="17" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" s="17" t="inlineStr">
+        <is>
+          <t>Impostazioni</t>
+        </is>
+      </c>
+      <c r="C61" s="17" t="inlineStr">
+        <is>
+          <t>test_impostazioni_05.py</t>
+        </is>
+      </c>
+      <c r="D61" s="17" t="inlineStr">
+        <is>
+          <t>test_posta_indesiderata</t>
+        </is>
+      </c>
+      <c r="E61" s="17" t="inlineStr">
+        <is>
+          <t>Verifica la sezione Posta indesiderata e il blocco di un mittente.</t>
+        </is>
+      </c>
+      <c r="F61" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare a Impostazioni &gt; Account e sicurezza &gt; Posta indesiderata.
+3. Scattare screenshot.
+4. Verificare che la sezione sia caricata.
+5. Aggiungere un indirizzo email alla lista di blocco.
+6. Verificare che l'indirizzo sia nella lista.
+7. Rimuovere l'indirizzo (cleanup).</t>
+        </is>
+      </c>
+      <c r="G61" s="17" t="inlineStr">
+        <is>
+          <t>La sezione Posta indesiderata è accessibile; è possibile aggiungere e rimuovere indirizzi dalla lista di blocco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="68.8" customHeight="1">
+      <c r="A62" s="23" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" s="23" t="inlineStr">
+        <is>
+          <t>Impostazioni</t>
+        </is>
+      </c>
+      <c r="C62" s="23" t="inlineStr">
+        <is>
+          <t>test_impostazioni_06.py</t>
+        </is>
+      </c>
+      <c r="D62" s="23" t="inlineStr">
+        <is>
+          <t>test_impostazioni_cestino</t>
+        </is>
+      </c>
+      <c r="E62" s="23" t="inlineStr">
+        <is>
+          <t>Verifica le opzioni di configurazione del Cestino nelle Impostazioni.</t>
+        </is>
+      </c>
+      <c r="F62" s="23" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare direttamente a /new/settings/messages-writing/empty-trash.
+3. Attendere l'h1 'Cestino' visibile.
+4. Verificare la presenza di testo relativo allo svuotamento/eliminazione automatica.
+5. Verificare la presenza di almeno un'opzione di configurazione (select/radio/checkbox).
+6. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="G62" s="23" t="inlineStr">
+        <is>
+          <t>La sezione Cestino nelle Impostazioni è accessibile e le opzioni di configurazione sono presenti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="50" customHeight="1">
+      <c r="A63" s="17" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" s="17" t="inlineStr">
+        <is>
+          <t>Impostazioni</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="inlineStr">
+        <is>
+          <t>test_impostazioni_07.py</t>
+        </is>
+      </c>
+      <c r="D63" s="17" t="inlineStr">
+        <is>
+          <t>test_storico_accessi</t>
+        </is>
+      </c>
+      <c r="E63" s="17" t="inlineStr">
+        <is>
+          <t>Verifica l'accesso e la visualizzazione dello storico degli accessi alla casella PEL.</t>
+        </is>
+      </c>
+      <c r="F63" s="17" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare direttamente a /new/settings/account-security/access-history.
+3. Scattare screenshot.
+4. Verificare che l'URL contenga 'access-history' o 'account-security' (assert).</t>
+        </is>
+      </c>
+      <c r="G63" s="17" t="inlineStr">
+        <is>
+          <t>La pagina Storico accessi è raggiungibile correttamente.</t>
         </is>
       </c>
     </row>
@@ -1899,6 +3902,947 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="55" t="inlineStr">
+        <is>
+          <t>MODULO: MESSAGGI – 25 Casi di Test (27 su PEC, 2 esclusi: Ricevute RA/RD)</t>
+        </is>
+      </c>
+      <c r="B1" s="55" t="n"/>
+      <c r="C1" s="55" t="n"/>
+      <c r="D1" s="55" t="n"/>
+      <c r="E1" s="55" t="n"/>
+      <c r="F1" s="55" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="81" t="inlineStr">
+        <is>
+          <t>File / Funzione</t>
+        </is>
+      </c>
+      <c r="C2" s="81" t="inlineStr">
+        <is>
+          <t>Descrizione</t>
+        </is>
+      </c>
+      <c r="D2" s="81" t="inlineStr">
+        <is>
+          <t>Passi</t>
+        </is>
+      </c>
+      <c r="E2" s="81" t="inlineStr">
+        <is>
+          <t>Risultato Atteso</t>
+        </is>
+      </c>
+      <c r="F2" s="81" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="98.80952380952381" customHeight="1">
+      <c r="A3" s="82" t="n">
+        <v>18</v>
+      </c>
+      <c r="B3" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_01.py
+test_messaggio_con_allegato</t>
+        </is>
+      </c>
+      <c r="C3" s="58" t="inlineStr">
+        <is>
+          <t>Verifica l'invio di un messaggio PEL con allegato e la sua corretta visualizzazione.</t>
+        </is>
+      </c>
+      <c r="D3" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire l'indirizzo del destinatario principale.
+4. Inserire oggetto e corpo del messaggio.
+5. Allegare un file PDF tramite il pulsante allegati.
+6. Inviare il messaggio.
+7. Attendere la ricezione nella cartella In arrivo.
+8. Aprire il messaggio ricevuto.
+9. Scattare screenshot.
+10. Verificare la presenza dell'allegato nel messaggio (assert).</t>
+        </is>
+      </c>
+      <c r="E3" s="58" t="inlineStr">
+        <is>
+          <t>Il messaggio è presente in In arrivo. L'allegato è visibile all'interno del messaggio ricevuto.</t>
+        </is>
+      </c>
+      <c r="F3" s="58" t="n"/>
+    </row>
+    <row r="4" ht="85.71428571428571" customHeight="1">
+      <c r="A4" s="83" t="n">
+        <v>19</v>
+      </c>
+      <c r="B4" s="51" t="inlineStr">
+        <is>
+          <t>test_messaggi_02.py
+test_messaggio_inoltrato</t>
+        </is>
+      </c>
+      <c r="C4" s="51" t="inlineStr">
+        <is>
+          <t>Verifica l'inoltro di un messaggio PEL ricevuto.</t>
+        </is>
+      </c>
+      <c r="D4" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare un messaggio a se stessi con oggetto univoco.
+3. Attendere la ricezione del messaggio.
+4. Aprire il messaggio ricevuto.
+5. Cliccare il pulsante 'Inoltra'.
+6. Inserire il destinatario dell'inoltro.
+7. Inviare il messaggio inoltrato.
+8. Scattare screenshot.
+9. Verificare la comparsa del toast di conferma (assert).</t>
+        </is>
+      </c>
+      <c r="E4" s="51" t="inlineStr">
+        <is>
+          <t>Il messaggio inoltrato è inviato correttamente. Il toast di conferma è visibile. L'oggetto contiene il prefisso di inoltro.</t>
+        </is>
+      </c>
+      <c r="F4" s="51" t="n"/>
+    </row>
+    <row r="5" ht="72.61904761904762" customHeight="1">
+      <c r="A5" s="82" t="n">
+        <v>20</v>
+      </c>
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_03.py
+test_messaggio_in_bozza</t>
+        </is>
+      </c>
+      <c r="C5" s="58" t="inlineStr">
+        <is>
+          <t>Verifica il salvataggio di un messaggio come bozza e il successivo invio.</t>
+        </is>
+      </c>
+      <c r="D5" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire destinatario, oggetto e corpo.
+4. Cliccare 'Salva bozza' (o chiudere la finestra senza inviare).
+5. Navigare nella cartella Bozze.
+6. Verificare che la bozza sia presente.
+7. Aprire la bozza e inviarla.
+8. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="E5" s="58" t="inlineStr">
+        <is>
+          <t>La bozza è visibile nella cartella Bozze. Dopo l'invio, la bozza non è più presente nella cartella Bozze.</t>
+        </is>
+      </c>
+      <c r="F5" s="58" t="inlineStr">
+        <is>
+          <t>Su PEL il pulsante di chiusura del dialog messaggio ha 2 elementi corrispondenti: selettore con .first per evitare strict-mode violation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="66.19047619047619" customHeight="1">
+      <c r="A6" s="83" t="n">
+        <v>21</v>
+      </c>
+      <c r="B6" s="51" t="inlineStr">
+        <is>
+          <t>test_messaggi_04.py
+test_messaggio_importato</t>
+        </is>
+      </c>
+      <c r="C6" s="51" t="inlineStr">
+        <is>
+          <t>Verifica l'importazione di messaggi da file nella casella PEL.</t>
+        </is>
+      </c>
+      <c r="D6" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Aprire il menu di importazione messaggi.
+3. Selezionare il file da importare.
+4. Avviare il processo di importazione.
+5. Attendere il completamento dell'importazione.
+6. Scattare screenshot.
+7. Verificare il messaggio di conferma (assert).</t>
+        </is>
+      </c>
+      <c r="E6" s="51" t="inlineStr">
+        <is>
+          <t>Il processo di importazione si completa senza errori. Viene mostrato un messaggio di successo o conferma.</t>
+        </is>
+      </c>
+      <c r="F6" s="51" t="inlineStr">
+        <is>
+          <t>Assert sul toast allargato per accettare anche 'nuovi messaggi' (plurale), oltre al singolare 'nuovo messaggio'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="81.66666666666666" customHeight="1">
+      <c r="A7" s="82" t="n">
+        <v>22</v>
+      </c>
+      <c r="B7" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_05.py
+test_cartella</t>
+        </is>
+      </c>
+      <c r="C7" s="58" t="inlineStr">
+        <is>
+          <t>Verifica la creazione, la modifica e l'eliminazione di una cartella personalizzata.</t>
+        </is>
+      </c>
+      <c r="D7" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare una nuova cartella con nome univoco.
+3. Verificare il toast di conferma della creazione.
+4. Rinominare la cartella con un nuovo nome.
+5. Verificare il toast di conferma della modifica.
+6. Eliminare la cartella.
+7. Scattare screenshot.
+8. Verificare il toast di conferma dell'eliminazione (assert).</t>
+        </is>
+      </c>
+      <c r="E7" s="58" t="inlineStr">
+        <is>
+          <t>La cartella è creata, rinominata ed eliminata con successo. Per ogni operazione compare un toast di conferma.</t>
+        </is>
+      </c>
+      <c r="F7" s="58" t="inlineStr">
+        <is>
+          <t>Usa trova_cartella_sidebar(): la sidebar cartelle è a virtual-scroll (Angular CDK), serve scroll reale via mouse.wheel().</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="85.95238095238095" customHeight="1">
+      <c r="A8" s="83" t="n">
+        <v>23</v>
+      </c>
+      <c r="B8" s="51" t="inlineStr">
+        <is>
+          <t>test_messaggi_06.py
+test_ripristino_messaggi</t>
+        </is>
+      </c>
+      <c r="C8" s="51" t="inlineStr">
+        <is>
+          <t>Verifica il ripristino di messaggi dal cestino alla cartella In arrivo.</t>
+        </is>
+      </c>
+      <c r="D8" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Spostare un messaggio nel cestino.
+3. Navigare nella cartella Cestino.
+4. Selezionare il/i messaggio/i da ripristinare.
+5. Cliccare 'Ripristina' o 'Sposta in In arrivo'.
+6. Verificare che i messaggi non siano più nel cestino.
+7. Scattare screenshot.
+8. Navigare in In arrivo e verificare la presenza dei messaggi (assert).</t>
+        </is>
+      </c>
+      <c r="E8" s="51" t="inlineStr">
+        <is>
+          <t>I messaggi ripristinati non sono più nel cestino e sono visibili nella cartella In arrivo.</t>
+        </is>
+      </c>
+      <c r="F8" s="51" t="n"/>
+    </row>
+    <row r="9" ht="81.66666666666666" customHeight="1">
+      <c r="A9" s="82" t="n">
+        <v>24</v>
+      </c>
+      <c r="B9" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_07.py
+test_messaggi_preferiti_pinnati</t>
+        </is>
+      </c>
+      <c r="C9" s="58" t="inlineStr">
+        <is>
+          <t>Verifica l'aggiunta di messaggi ai preferiti e la funzione 'Pinna messaggio'.</t>
+        </is>
+      </c>
+      <c r="D9" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Selezionare un messaggio dall'In arrivo.
+3. Aggiungere il messaggio ai preferiti (stella).
+4. Verificare che il messaggio compaia nella cartella Preferiti/Speciali.
+5. Selezionare un messaggio e cliccare 'Pinna messaggio'.
+6. Scattare screenshot.
+7. Verificare la presenza del messaggio pinnato (assert).</t>
+        </is>
+      </c>
+      <c r="E9" s="58" t="inlineStr">
+        <is>
+          <t>Il messaggio è aggiunto ai preferiti e compare nella sezione Preferiti. Il messaggio pinnato è visibile in cima alla lista.</t>
+        </is>
+      </c>
+      <c r="F9" s="58" t="n"/>
+    </row>
+    <row r="10" ht="83.80952380952381" customHeight="1">
+      <c r="A10" s="83" t="n">
+        <v>25</v>
+      </c>
+      <c r="B10" s="51" t="inlineStr">
+        <is>
+          <t>test_messaggi_08.py
+test_etichetta</t>
+        </is>
+      </c>
+      <c r="C10" s="51" t="inlineStr">
+        <is>
+          <t>Verifica la creazione di un'etichetta, la sua applicazione ai messaggi e l'eliminazione.</t>
+        </is>
+      </c>
+      <c r="D10" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Aprire le impostazioni etichette.
+3. Creare una nuova etichetta con nome univoco e colore.
+4. Tornare in In arrivo e selezionare un messaggio.
+5. Applicare l'etichetta appena creata al messaggio.
+6. Verificare che l'etichetta sia visibile sul messaggio.
+7. Scattare screenshot.
+8. Eliminare l'etichetta (cleanup).</t>
+        </is>
+      </c>
+      <c r="E10" s="51" t="inlineStr">
+        <is>
+          <t>L'etichetta è creata e applicata con successo al messaggio. Dopo l'eliminazione dell'etichetta, essa non è più visibile.</t>
+        </is>
+      </c>
+      <c r="F10" s="51" t="n"/>
+    </row>
+    <row r="11" ht="81.19047619047619" customHeight="1">
+      <c r="A11" s="82" t="n">
+        <v>26</v>
+      </c>
+      <c r="B11" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_09.py
+test_segna_come_letto_da_leggere</t>
+        </is>
+      </c>
+      <c r="C11" s="58" t="inlineStr">
+        <is>
+          <t>Verifica le funzioni 'Segna come letto' e 'Segna come da leggere' sui messaggi.</t>
+        </is>
+      </c>
+      <c r="D11" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Selezionare un messaggio non letto dall'In arrivo.
+3. Cliccare 'Segna come letto'.
+4. Verificare che il messaggio non sia più in grassetto (letto).
+5. Cliccare 'Segna come da leggere' sullo stesso messaggio.
+6. Scattare screenshot.
+7. Verificare che il messaggio torni in grassetto (non letto, assert).</t>
+        </is>
+      </c>
+      <c r="E11" s="58" t="inlineStr">
+        <is>
+          <t>I pulsanti 'Segna come letto' e 'Segna come da leggere' sono visibili e funzionanti. Lo stato del messaggio cambia correttamente.</t>
+        </is>
+      </c>
+      <c r="F11" s="58" t="n"/>
+    </row>
+    <row r="12" ht="83.33333333333333" customHeight="1">
+      <c r="A12" s="83" t="n">
+        <v>27</v>
+      </c>
+      <c r="B12" s="51" t="inlineStr">
+        <is>
+          <t>test_messaggi_10.py
+test_messaggio_alta_priorita</t>
+        </is>
+      </c>
+      <c r="C12" s="51" t="inlineStr">
+        <is>
+          <t>Verifica l'invio e la ricezione di un messaggio con priorità alta.</t>
+        </is>
+      </c>
+      <c r="D12" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire destinatario, oggetto e corpo.
+4. Impostare la priorità del messaggio su 'Alta'.
+5. Inviare il messaggio.
+6. Attendere la ricezione in In arrivo.
+7. Aprire il messaggio ricevuto.
+8. Scattare screenshot.
+9. Verificare la presenza dell'indicatore di alta priorità (assert).</t>
+        </is>
+      </c>
+      <c r="E12" s="51" t="inlineStr">
+        <is>
+          <t>Il messaggio è ricevuto con l'indicatore di alta priorità visibile (simbolo '!' o equivalente).</t>
+        </is>
+      </c>
+      <c r="F12" s="51" t="n"/>
+    </row>
+    <row r="13" ht="73.09523809523809" customHeight="1">
+      <c r="A13" s="82" t="n">
+        <v>28</v>
+      </c>
+      <c r="B13" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_11.py
+test_risposta_messaggio</t>
+        </is>
+      </c>
+      <c r="C13" s="58" t="inlineStr">
+        <is>
+          <t>Verifica la risposta a un messaggio PEL ricevuto.</t>
+        </is>
+      </c>
+      <c r="D13" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare un messaggio a se stessi.
+3. Attendere la ricezione del messaggio.
+4. Aprire il messaggio ricevuto.
+5. Cliccare il pulsante 'Rispondi'.
+6. Verificare che la finestra di risposta sia aperta con 'Re:' nell'oggetto.
+7. Inviare la risposta.
+8. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="E13" s="58" t="inlineStr">
+        <is>
+          <t>La finestra di risposta si apre correttamente. L'oggetto contiene il prefisso 'Re:'. La risposta viene inviata con successo.</t>
+        </is>
+      </c>
+      <c r="F13" s="58" t="n"/>
+    </row>
+    <row r="14" ht="61.90476190476191" customHeight="1">
+      <c r="A14" s="83" t="n">
+        <v>29</v>
+      </c>
+      <c r="B14" s="51" t="inlineStr">
+        <is>
+          <t>test_messaggi_12.py
+test_invio_messaggio_semplice</t>
+        </is>
+      </c>
+      <c r="C14" s="51" t="inlineStr">
+        <is>
+          <t>Verifica l'invio di un messaggio PEL semplice senza allegati.</t>
+        </is>
+      </c>
+      <c r="D14" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire l'indirizzo del destinatario.
+4. Inserire oggetto e corpo del messaggio.
+5. Cliccare 'Invia'.
+6. Scattare screenshot.
+7. Verificare la comparsa del toast di conferma invio (assert).</t>
+        </is>
+      </c>
+      <c r="E14" s="51" t="inlineStr">
+        <is>
+          <t>Il messaggio è inviato con successo. Appare un toast di conferma dell'invio.</t>
+        </is>
+      </c>
+      <c r="F14" s="51" t="n"/>
+    </row>
+    <row r="15" ht="91.9047619047619" customHeight="1">
+      <c r="A15" s="82" t="n">
+        <v>30</v>
+      </c>
+      <c r="B15" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_13.py
+test_risposta_a_tutti</t>
+        </is>
+      </c>
+      <c r="C15" s="58" t="inlineStr">
+        <is>
+          <t>Verifica la funzione 'Rispondi a tutti' su un messaggio ricevuto.</t>
+        </is>
+      </c>
+      <c r="D15" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare un messaggio a se stessi.
+3. Attendere la ricezione del messaggio.
+4. Aprire il messaggio ricevuto.
+5. Cliccare il pulsante 'Rispondi a tutti'.
+6. Verificare che la finestra di risposta sia aperta con 'Re:' nell'oggetto.
+7. Verificare che tutti i destinatari originali siano inclusi.
+8. Inviare la risposta a tutti.
+9. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="E15" s="58" t="inlineStr">
+        <is>
+          <t>La finestra di risposta si apre con l'oggetto 'Re: ...' e tutti i destinatari originali inclusi. La risposta viene inviata con successo.</t>
+        </is>
+      </c>
+      <c r="F15" s="58" t="n"/>
+    </row>
+    <row r="16" ht="75.95238095238095" customHeight="1">
+      <c r="A16" s="83" t="n">
+        <v>31</v>
+      </c>
+      <c r="B16" s="51" t="inlineStr">
+        <is>
+          <t>test_messaggi_14.py
+test_elimina_messaggio</t>
+        </is>
+      </c>
+      <c r="C16" s="51" t="inlineStr">
+        <is>
+          <t>Verifica l'eliminazione di un messaggio e la sua presenza nel cestino.</t>
+        </is>
+      </c>
+      <c r="D16" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare un messaggio a se stessi con oggetto univoco.
+3. Attendere la ricezione del messaggio.
+4. Selezionare il messaggio e cliccare 'Elimina'.
+5. Navigare nella cartella Cestino.
+6. Scattare screenshot.
+7. Verificare che il messaggio eliminato sia presente nel cestino (assert).</t>
+        </is>
+      </c>
+      <c r="E16" s="51" t="inlineStr">
+        <is>
+          <t>Il messaggio eliminato non è più in In arrivo ma è visibile nella cartella Cestino.</t>
+        </is>
+      </c>
+      <c r="F16" s="51" t="n"/>
+    </row>
+    <row r="17" ht="102.8571428571428" customHeight="1">
+      <c r="A17" s="82" t="n">
+        <v>32</v>
+      </c>
+      <c r="B17" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_15.py
+test_sposta_messaggio_in_cartella</t>
+        </is>
+      </c>
+      <c r="C17" s="58" t="inlineStr">
+        <is>
+          <t>Verifica lo spostamento di un messaggio in una cartella personalizzata.</t>
+        </is>
+      </c>
+      <c r="D17" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare una nuova cartella con nome univoco.
+3. Inviare un messaggio a se stessi.
+4. Attendere la ricezione del messaggio.
+5. Selezionare il messaggio e cliccare 'Sposta in...'.
+6. Selezionare la cartella di destinazione.
+7. Verificare che il messaggio non sia più in In arrivo.
+8. Scattare screenshot.
+9. Navigare nella cartella di destinazione e verificare la presenza del messaggio (assert).</t>
+        </is>
+      </c>
+      <c r="E17" s="58" t="inlineStr">
+        <is>
+          <t>Il messaggio è spostato correttamente nella cartella di destinazione e non è più visibile in In arrivo.</t>
+        </is>
+      </c>
+      <c r="F17" s="58" t="inlineStr">
+        <is>
+          <t>Usa trova_cartella_sidebar() per individuare la cartella di destinazione nella lista a virtual-scroll.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="91.42857142857143" customHeight="1">
+      <c r="A18" s="83" t="n">
+        <v>33</v>
+      </c>
+      <c r="B18" s="51" t="inlineStr">
+        <is>
+          <t>test_messaggi_16.py
+test_copia_messaggio_in_cartella</t>
+        </is>
+      </c>
+      <c r="C18" s="51" t="inlineStr">
+        <is>
+          <t>Verifica la copia di un messaggio in una cartella personalizzata.</t>
+        </is>
+      </c>
+      <c r="D18" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare una nuova cartella con nome univoco.
+3. Aprire un messaggio esistente in In arrivo.
+4. Selezionare 'Copia in...' dal menu azioni.
+5. Selezionare la cartella di destinazione.
+6. Verificare che il messaggio originale sia ancora in In arrivo.
+7. Scattare screenshot.
+8. Navigare nella cartella di destinazione e verificare la copia (assert).</t>
+        </is>
+      </c>
+      <c r="E18" s="51" t="inlineStr">
+        <is>
+          <t>Il messaggio è copiato nella cartella di destinazione. Il messaggio originale rimane in In arrivo.</t>
+        </is>
+      </c>
+      <c r="F18" s="51" t="n"/>
+    </row>
+    <row r="19" ht="72.14285714285714" customHeight="1">
+      <c r="A19" s="82" t="n">
+        <v>34</v>
+      </c>
+      <c r="B19" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_17.py
+test_ricerca_messaggi</t>
+        </is>
+      </c>
+      <c r="C19" s="58" t="inlineStr">
+        <is>
+          <t>Verifica la funzione di ricerca messaggi nella casella PEL.</t>
+        </is>
+      </c>
+      <c r="D19" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare un messaggio a se stessi con oggetto univoco.
+3. Attendere la ricezione del messaggio.
+4. Inserire il testo univoco nella barra di ricerca.
+5. Avviare la ricerca.
+6. Scattare screenshot.
+7. Verificare che il messaggio cercato appaia nei risultati (assert).</t>
+        </is>
+      </c>
+      <c r="E19" s="58" t="inlineStr">
+        <is>
+          <t>Il messaggio con l'oggetto univoco è trovato e visibile nei risultati di ricerca.</t>
+        </is>
+      </c>
+      <c r="F19" s="58" t="n"/>
+    </row>
+    <row r="20" ht="75.23809523809524" customHeight="1">
+      <c r="A20" s="83" t="n">
+        <v>35</v>
+      </c>
+      <c r="B20" s="51" t="inlineStr">
+        <is>
+          <t>test_messaggi_18.py
+test_filtri_inbox</t>
+        </is>
+      </c>
+      <c r="C20" s="51" t="inlineStr">
+        <is>
+          <t>Verifica la presenza e il funzionamento del filtro messaggi (Tutti/Letti/Da leggere) nella lista In arrivo.</t>
+        </is>
+      </c>
+      <c r="D20" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Attendere che i messaggi siano visibili in In arrivo.
+3. Individuare il filtro 'Letti' tra i tab aru-chip in alto alla lista.
+4. Cliccare il filtro 'Letti'.
+5. Scattare screenshot.
+6. Verificare che l'URL rifletta il quick-filter applicato (parametro mail_quickFilter, assert).</t>
+        </is>
+      </c>
+      <c r="E20" s="51" t="inlineStr">
+        <is>
+          <t>Il filtro 'Letti' è visibile e cliccabile. Dopo il click l'URL contiene il parametro 'mail_quickFilter', confermando che il filtro è stato applicato.</t>
+        </is>
+      </c>
+      <c r="F20" s="51" t="inlineStr">
+        <is>
+          <t>Riscritto rispetto a PEC: su PEL il filtro è una fila di tab aru-chip (Tutti/Letti/Da leggere), non un dropdown aru-input-select. Il selettore generico su 'Letti' matcherebbe anche il bottone toolbar 'Segna tutti come già letti': serve scoping sulla classe .aru-chip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="68.80952380952381" customHeight="1">
+      <c r="A21" s="82" t="n">
+        <v>36</v>
+      </c>
+      <c r="B21" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_19.py
+test_invio_messaggio_con_cc</t>
+        </is>
+      </c>
+      <c r="C21" s="58" t="inlineStr">
+        <is>
+          <t>Verifica l'invio di un messaggio PEL con destinatario in copia (CC).</t>
+        </is>
+      </c>
+      <c r="D21" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire l'indirizzo del destinatario principale.
+4. Aggiungere un destinatario in CC.
+5. Inserire oggetto e corpo del messaggio.
+6. Cliccare 'Invia'.
+7. Scattare screenshot.
+8. Verificare la conferma di invio (assert).</t>
+        </is>
+      </c>
+      <c r="E21" s="58" t="inlineStr">
+        <is>
+          <t>Il messaggio è inviato con successo con entrambi i destinatari (To e CC). Appare il toast di conferma.</t>
+        </is>
+      </c>
+      <c r="F21" s="58" t="inlineStr">
+        <is>
+          <t>Su PEL il bottone è etichettato 'CC/CCn' (CC e CCN combinati in un unico pulsante), non solo 'CC' come su PEC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="100.4761904761905" customHeight="1">
+      <c r="A22" s="83" t="n">
+        <v>37</v>
+      </c>
+      <c r="B22" s="51" t="inlineStr">
+        <is>
+          <t>test_messaggi_20.py
+test_scarica_allegato_ricevuto</t>
+        </is>
+      </c>
+      <c r="C22" s="51" t="inlineStr">
+        <is>
+          <t>Verifica il download di un allegato da un messaggio PEL ricevuto.</t>
+        </is>
+      </c>
+      <c r="D22" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare a se stessi un messaggio con allegato PDF.
+3. Attendere la ricezione del messaggio.
+4. Aprire il messaggio ricevuto.
+5. Cliccare sul pulsante di download dell'allegato.
+6. Gestire il download tramite Playwright expect_download.
+7. Salvare il file nella cartella test-results.
+8. Scattare screenshot.
+9. Verificare che il file scaricato esista e abbia dimensione &gt; 0 (assert).</t>
+        </is>
+      </c>
+      <c r="E22" s="51" t="inlineStr">
+        <is>
+          <t>Il file allegato viene scaricato correttamente. Il file esiste nella directory di destinazione e ha dimensione maggiore di 0 byte.</t>
+        </is>
+      </c>
+      <c r="F22" s="51" t="n"/>
+    </row>
+    <row r="23" ht="75.47619047619047" customHeight="1">
+      <c r="A23" s="82" t="n">
+        <v>38</v>
+      </c>
+      <c r="B23" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_21.py
+test_salva_e_usa_modello</t>
+        </is>
+      </c>
+      <c r="C23" s="58" t="inlineStr">
+        <is>
+          <t>Verifica il salvataggio di un messaggio come modello e il suo successivo utilizzo.</t>
+        </is>
+      </c>
+      <c r="D23" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire oggetto e corpo del messaggio modello.
+4. Salvare come modello invece di inviare.
+5. Navigare nella cartella Modelli.
+6. Verificare che il modello sia presente.
+7. Aprire il modello e inviarlo come nuovo messaggio.
+8. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="E23" s="58" t="inlineStr">
+        <is>
+          <t>Il modello è salvato e visibile nella cartella Modelli. Può essere aperto e utilizzato per inviare un nuovo messaggio.</t>
+        </is>
+      </c>
+      <c r="F23" s="58" t="n"/>
+    </row>
+    <row r="24" ht="71.42857142857143" customHeight="1">
+      <c r="A24" s="83" t="n">
+        <v>39</v>
+      </c>
+      <c r="B24" s="51" t="inlineStr">
+        <is>
+          <t>test_messaggi_22.py
+test_verifica_cartella_inviati</t>
+        </is>
+      </c>
+      <c r="C24" s="51" t="inlineStr">
+        <is>
+          <t>Verifica che i messaggi inviati siano presenti nella cartella Inviati.</t>
+        </is>
+      </c>
+      <c r="D24" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare un messaggio con oggetto univoco.
+3. Attendere la conferma di invio.
+4. Navigare nella cartella Inviati.
+5. Cercare il messaggio con l'oggetto univoco.
+6. Scattare screenshot.
+7. Verificare che il messaggio sia presente con il corretto oggetto (assert).</t>
+        </is>
+      </c>
+      <c r="E24" s="51" t="inlineStr">
+        <is>
+          <t>Il messaggio inviato è visibile nella cartella Inviati con l'oggetto corretto.</t>
+        </is>
+      </c>
+      <c r="F24" s="51" t="n"/>
+    </row>
+    <row r="25" ht="80.47619047619047" customHeight="1">
+      <c r="A25" s="82" t="n">
+        <v>40</v>
+      </c>
+      <c r="B25" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_25.py
+test_invio_allegati_multipli</t>
+        </is>
+      </c>
+      <c r="C25" s="58" t="inlineStr">
+        <is>
+          <t>Verifica l'invio di un messaggio con allegati multipli.</t>
+        </is>
+      </c>
+      <c r="D25" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire destinatario, oggetto e corpo.
+4. Cliccare il pulsante allegati e selezionare il primo file.
+5. Aggiungere un secondo allegato.
+6. Verificare che almeno 2 allegati siano visibili nella finestra di composizione.
+7. Inviare il messaggio.
+8. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="E25" s="58" t="inlineStr">
+        <is>
+          <t>Almeno 2 allegati sono visibili nella finestra di composizione prima dell'invio. Il messaggio viene inviato con successo.</t>
+        </is>
+      </c>
+      <c r="F25" s="58" t="n"/>
+    </row>
+    <row r="26" ht="99.28571428571428" customHeight="1">
+      <c r="A26" s="83" t="n">
+        <v>41</v>
+      </c>
+      <c r="B26" s="51" t="inlineStr">
+        <is>
+          <t>test_messaggi_26.py
+test_selezione_multipla_batch</t>
+        </is>
+      </c>
+      <c r="C26" s="51" t="inlineStr">
+        <is>
+          <t>Verifica la selezione multipla di messaggi e la comparsa della toolbar azioni batch.</t>
+        </is>
+      </c>
+      <c r="D26" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Inviare 2 messaggi a se stessi con oggetti univoci.
+3. Attendere la ricezione di entrambi in In arrivo.
+4. Passare il mouse sulla prima riga messaggio per rivelare il checkbox.
+5. Selezionare il checkbox della prima riga.
+6. Passare il mouse sulla seconda riga e selezionare il suo checkbox.
+7. Scattare screenshot.
+8. Verificare la comparsa della toolbar azioni batch (assert).</t>
+        </is>
+      </c>
+      <c r="E26" s="51" t="inlineStr">
+        <is>
+          <t>Dopo la selezione di almeno 2 messaggi, la toolbar delle azioni batch è visibile con i relativi pulsanti.</t>
+        </is>
+      </c>
+      <c r="F26" s="51" t="n"/>
+    </row>
+    <row r="27" ht="83.09523809523809" customHeight="1">
+      <c r="A27" s="82" t="n">
+        <v>42</v>
+      </c>
+      <c r="B27" s="58" t="inlineStr">
+        <is>
+          <t>test_messaggi_27.py
+test_anomalia_invio_non_pec</t>
+        </is>
+      </c>
+      <c r="C27" s="58" t="inlineStr">
+        <is>
+          <t>Verifica che l'invio a un indirizzo non-PEC generi una notifica di anomalia.</t>
+        </is>
+      </c>
+      <c r="D27" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Cliccare 'Nuovo messaggio'.
+3. Inserire un indirizzo email non-PEC come destinatario.
+4. Inserire oggetto e corpo del messaggio.
+5. Inviare il messaggio.
+6. Attendere la ricezione della notifica di anomalia.
+7. Scattare screenshot.
+8. Verificare la presenza della notifica nell'inbox o come avviso UI (assert).</t>
+        </is>
+      </c>
+      <c r="E27" s="58" t="inlineStr">
+        <is>
+          <t>Viene generata e ricevuta una notifica di anomalia per l'invio a un indirizzo non-PEC.</t>
+        </is>
+      </c>
+      <c r="F27" s="58" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2419,7 +5363,868 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="55" t="inlineStr">
+        <is>
+          <t>MODULO: CONTATTI – 10 Casi di Test</t>
+        </is>
+      </c>
+      <c r="B1" s="55" t="n"/>
+      <c r="C1" s="55" t="n"/>
+      <c r="D1" s="55" t="n"/>
+      <c r="E1" s="55" t="n"/>
+      <c r="F1" s="55" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="81" t="inlineStr">
+        <is>
+          <t>File / Funzione</t>
+        </is>
+      </c>
+      <c r="C2" s="81" t="inlineStr">
+        <is>
+          <t>Descrizione</t>
+        </is>
+      </c>
+      <c r="D2" s="81" t="inlineStr">
+        <is>
+          <t>Passi</t>
+        </is>
+      </c>
+      <c r="E2" s="81" t="inlineStr">
+        <is>
+          <t>Risultato Atteso</t>
+        </is>
+      </c>
+      <c r="F2" s="81" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="67.61904761904762" customHeight="1">
+      <c r="A3" s="82" t="n">
+        <v>43</v>
+      </c>
+      <c r="B3" s="58" t="inlineStr">
+        <is>
+          <t>test_contatti_01.py
+test_aggiungere_nuovo_contatto</t>
+        </is>
+      </c>
+      <c r="C3" s="58" t="inlineStr">
+        <is>
+          <t>Verifica la creazione di un nuovo contatto nella rubrica della casella PEL.</t>
+        </is>
+      </c>
+      <c r="D3" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare nella sezione Contatti.
+3. Cliccare 'Nuovo contatto'.
+4. Inserire nome, cognome e indirizzo email.
+5. Salvare il contatto.
+6. Verificare la presenza del contatto nella rubrica.
+7. Scattare screenshot.
+8. Eliminare il contatto (cleanup).</t>
+        </is>
+      </c>
+      <c r="E3" s="58" t="inlineStr">
+        <is>
+          <t>Il contatto è creato e visibile nella rubrica con nome, cognome e email corretti. Può essere eliminato correttamente.</t>
+        </is>
+      </c>
+      <c r="F3" s="58" t="n"/>
+    </row>
+    <row r="4" ht="79.28571428571428" customHeight="1">
+      <c r="A4" s="83" t="n">
+        <v>44</v>
+      </c>
+      <c r="B4" s="51" t="inlineStr">
+        <is>
+          <t>test_contatti_02.py
+test_aggiungere_nuovo_gruppo</t>
+        </is>
+      </c>
+      <c r="C4" s="51" t="inlineStr">
+        <is>
+          <t>Verifica la creazione di un gruppo contatti e l'aggiunta di contatti al gruppo.</t>
+        </is>
+      </c>
+      <c r="D4" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare nella sezione Contatti.
+3. Cliccare 'Nuovo gruppo'.
+4. Inserire il nome del gruppo.
+5. Salvare il gruppo.
+6. Aggiungere uno o più contatti al gruppo.
+7. Verificare che il gruppo sia visibile nella sidebar.
+8. Scattare screenshot.
+9. Verificare che i contatti siano nel gruppo (assert).</t>
+        </is>
+      </c>
+      <c r="E4" s="51" t="inlineStr">
+        <is>
+          <t>Il gruppo è creato e visibile nella sidebar. I contatti aggiunti sono visibili nel gruppo.</t>
+        </is>
+      </c>
+      <c r="F4" s="51" t="n"/>
+    </row>
+    <row r="5" ht="80.95238095238095" customHeight="1">
+      <c r="A5" s="82" t="n">
+        <v>45</v>
+      </c>
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>test_contatti_03.py
+test_esporta_contatti</t>
+        </is>
+      </c>
+      <c r="C5" s="58" t="inlineStr">
+        <is>
+          <t>Verifica l'esportazione della rubrica contatti in formato CSV.</t>
+        </is>
+      </c>
+      <c r="D5" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare nella sezione Contatti.
+3. Aprire il menu Opzioni della rubrica.
+4. Selezionare 'Esporta rubrica'.
+5. Gestire il download del file tramite Playwright expect_download.
+6. Verificare che il file CSV sia scaricato.
+7. Scattare screenshot.
+8. Verificare che il file abbia dimensione &gt; 0 (assert).</t>
+        </is>
+      </c>
+      <c r="E5" s="58" t="inlineStr">
+        <is>
+          <t>Il file CSV della rubrica è scaricato correttamente con dimensione maggiore di 0 byte.</t>
+        </is>
+      </c>
+      <c r="F5" s="58" t="n"/>
+    </row>
+    <row r="6" ht="69.52380952380952" customHeight="1">
+      <c r="A6" s="83" t="n">
+        <v>46</v>
+      </c>
+      <c r="B6" s="51" t="inlineStr">
+        <is>
+          <t>test_contatti_04.py
+test_importa_contatti</t>
+        </is>
+      </c>
+      <c r="C6" s="51" t="inlineStr">
+        <is>
+          <t>Verifica l'importazione di contatti da un file CSV nella rubrica PEL.</t>
+        </is>
+      </c>
+      <c r="D6" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare nella sezione Contatti.
+3. Cliccare 'Importa'.
+4. Selezionare il file CSV di test tramite il file picker.
+5. Confermare l'importazione.
+6. Verificare il messaggio di successo.
+7. Scattare screenshot.
+8. Eliminare i contatti importati (cleanup).</t>
+        </is>
+      </c>
+      <c r="E6" s="51" t="inlineStr">
+        <is>
+          <t>I contatti del file CSV sono importati con successo nella rubrica. Il messaggio di conferma è visibile.</t>
+        </is>
+      </c>
+      <c r="F6" s="51" t="n"/>
+    </row>
+    <row r="7" ht="83.33333333333333" customHeight="1">
+      <c r="A7" s="82" t="n">
+        <v>47</v>
+      </c>
+      <c r="B7" s="58" t="inlineStr">
+        <is>
+          <t>test_contatti_05.py
+test_modifica_contatto</t>
+        </is>
+      </c>
+      <c r="C7" s="58" t="inlineStr">
+        <is>
+          <t>Verifica la modifica dei dati di un contatto esistente nella rubrica.</t>
+        </is>
+      </c>
+      <c r="D7" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare un contatto da modificare.
+3. Cercare il contatto.
+4. Aprirlo e cliccare 'Modifica'.
+5. Cambiare il cognome con un valore nuovo univoco.
+6. Salvare le modifiche.
+7. Cercare il contatto con il nuovo cognome.
+8. Scattare screenshot.
+9. Verificare che il contatto sia trovato con i dati aggiornati (assert).</t>
+        </is>
+      </c>
+      <c r="E7" s="58" t="inlineStr">
+        <is>
+          <t>Il contatto è modificato correttamente. La ricerca con il nuovo cognome restituisce il contatto aggiornato.</t>
+        </is>
+      </c>
+      <c r="F7" s="58" t="n"/>
+    </row>
+    <row r="8" ht="67.85714285714286" customHeight="1">
+      <c r="A8" s="83" t="n">
+        <v>48</v>
+      </c>
+      <c r="B8" s="51" t="inlineStr">
+        <is>
+          <t>test_contatti_06.py
+test_elimina_contatto</t>
+        </is>
+      </c>
+      <c r="C8" s="51" t="inlineStr">
+        <is>
+          <t>Verifica l'eliminazione di un contatto dalla rubrica.</t>
+        </is>
+      </c>
+      <c r="D8" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare un contatto di test con nome univoco.
+3. Selezionare il contatto.
+4. Cliccare 'Elimina'.
+5. Confermare l'eliminazione.
+6. Cercare il contatto eliminato.
+7. Scattare screenshot.
+8. Verificare che non sia più presente nella rubrica (assert).</t>
+        </is>
+      </c>
+      <c r="E8" s="51" t="inlineStr">
+        <is>
+          <t>Il contatto eliminato non è più presente nella rubrica.</t>
+        </is>
+      </c>
+      <c r="F8" s="51" t="inlineStr">
+        <is>
+          <t>Include reload di sicurezza se la lista contatti non si aggiorna subito dopo la cancellazione lato server.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="63.57142857142857" customHeight="1">
+      <c r="A9" s="82" t="n">
+        <v>49</v>
+      </c>
+      <c r="B9" s="58" t="inlineStr">
+        <is>
+          <t>test_contatti_07.py
+test_ricerca_contatto</t>
+        </is>
+      </c>
+      <c r="C9" s="58" t="inlineStr">
+        <is>
+          <t>Verifica la ricerca di un contatto nella rubrica tramite la barra di ricerca.</t>
+        </is>
+      </c>
+      <c r="D9" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare un contatto con nome univoco.
+3. Inserire il nome univoco nella barra di ricerca.
+4. Avviare la ricerca.
+5. Verificare che il contatto cercato sia nei risultati.
+6. Scattare screenshot.
+7. Eliminare il contatto (cleanup).</t>
+        </is>
+      </c>
+      <c r="E9" s="58" t="inlineStr">
+        <is>
+          <t>Il contatto con il nome univoco è trovato e visibile nei risultati di ricerca della rubrica.</t>
+        </is>
+      </c>
+      <c r="F9" s="58" t="n"/>
+    </row>
+    <row r="10" ht="68.33333333333333" customHeight="1">
+      <c r="A10" s="83" t="n">
+        <v>50</v>
+      </c>
+      <c r="B10" s="51" t="inlineStr">
+        <is>
+          <t>test_contatti_08.py
+test_contatto_preferito</t>
+        </is>
+      </c>
+      <c r="C10" s="51" t="inlineStr">
+        <is>
+          <t>Verifica l'aggiunta di un contatto ai preferiti e la sua visualizzazione nella sezione Preferiti.</t>
+        </is>
+      </c>
+      <c r="D10" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Selezionare un contatto dalla rubrica.
+3. Cliccare il pulsante stella (preferito).
+4. Navigare nella sezione 'Contatti preferiti' nella sidebar.
+5. Verificare che il contatto sia presente.
+6. Scattare screenshot.
+7. Eliminare il contatto (cleanup).</t>
+        </is>
+      </c>
+      <c r="E10" s="51" t="inlineStr">
+        <is>
+          <t>Il contatto aggiunto ai preferiti è visibile nella sezione Contatti preferiti nella sidebar.</t>
+        </is>
+      </c>
+      <c r="F10" s="51" t="n"/>
+    </row>
+    <row r="11" ht="74.52380952380952" customHeight="1">
+      <c r="A11" s="82" t="n">
+        <v>51</v>
+      </c>
+      <c r="B11" s="58" t="inlineStr">
+        <is>
+          <t>test_contatti_09.py
+test_scrivi_email_da_contatto</t>
+        </is>
+      </c>
+      <c r="C11" s="58" t="inlineStr">
+        <is>
+          <t>Verifica l'apertura della finestra di composizione email direttamente da un contatto.</t>
+        </is>
+      </c>
+      <c r="D11" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare un contatto con email.
+3. Cercarlo nella rubrica.
+4. Cliccare il pulsante azione per scrivere email dal contatto.
+5. Verificare che la finestra di composizione si apra.
+6. Scattare screenshot.
+7. Chiudere il composer senza inviare.
+8. Eliminare il contatto (cleanup).</t>
+        </is>
+      </c>
+      <c r="E11" s="58" t="inlineStr">
+        <is>
+          <t>La finestra di composizione si apre correttamente a partire dal contatto selezionato.</t>
+        </is>
+      </c>
+      <c r="F11" s="58" t="n"/>
+    </row>
+    <row r="12" ht="68.57142857142857" customHeight="1">
+      <c r="A12" s="83" t="n">
+        <v>52</v>
+      </c>
+      <c r="B12" s="51" t="inlineStr">
+        <is>
+          <t>test_contatti_10.py
+test_elimina_gruppo</t>
+        </is>
+      </c>
+      <c r="C12" s="51" t="inlineStr">
+        <is>
+          <t>Verifica la creazione e l'eliminazione di un gruppo contatti.</t>
+        </is>
+      </c>
+      <c r="D12" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Creare un nuovo gruppo con nome univoco.
+3. Verificare la presenza del gruppo nella sidebar.
+4. Tasto destro sul gruppo ed Elimina.
+5. Confermare l'eliminazione.
+6. Scattare screenshot.
+7. Verificare che il gruppo non sia più nella sidebar (assert).</t>
+        </is>
+      </c>
+      <c r="E12" s="51" t="inlineStr">
+        <is>
+          <t>Il gruppo è eliminato correttamente e non è più visibile nella sidebar dei contatti.</t>
+        </is>
+      </c>
+      <c r="F12" s="51" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="55" t="inlineStr">
+        <is>
+          <t>MODULO: IMPOSTAZIONI – 7 Casi di Test</t>
+        </is>
+      </c>
+      <c r="B1" s="55" t="n"/>
+      <c r="C1" s="55" t="n"/>
+      <c r="D1" s="55" t="n"/>
+      <c r="E1" s="55" t="n"/>
+      <c r="F1" s="55" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="81" t="inlineStr">
+        <is>
+          <t>File / Funzione</t>
+        </is>
+      </c>
+      <c r="C2" s="81" t="inlineStr">
+        <is>
+          <t>Descrizione</t>
+        </is>
+      </c>
+      <c r="D2" s="81" t="inlineStr">
+        <is>
+          <t>Passi</t>
+        </is>
+      </c>
+      <c r="E2" s="81" t="inlineStr">
+        <is>
+          <t>Risultato Atteso</t>
+        </is>
+      </c>
+      <c r="F2" s="81" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60.71428571428571" customHeight="1">
+      <c r="A3" s="82" t="n">
+        <v>55</v>
+      </c>
+      <c r="B3" s="58" t="inlineStr">
+        <is>
+          <t>test_impostazioni_01.py
+test_crea_firma</t>
+        </is>
+      </c>
+      <c r="C3" s="58" t="inlineStr">
+        <is>
+          <t>Verifica la creazione di una firma email nella sezione Impostazioni.</t>
+        </is>
+      </c>
+      <c r="D3" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare direttamente a /new/settings/messages-writing/signatures.
+3. Verificare l'header 'Firme'.
+4. Cliccare il pulsante di creazione firma.
+5. Inserire nome e testo della firma.
+6. Salvare.
+7. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="E3" s="58" t="inlineStr">
+        <is>
+          <t>La pagina Firme si carica correttamente e il form di creazione firma è compilabile e salvabile.</t>
+        </is>
+      </c>
+      <c r="F3" s="58" t="n"/>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="83" t="n">
+        <v>56</v>
+      </c>
+      <c r="B4" s="51" t="inlineStr">
+        <is>
+          <t>test_impostazioni_02.py
+test_riquadro_di_lettura</t>
+        </is>
+      </c>
+      <c r="C4" s="51" t="inlineStr">
+        <is>
+          <t>Verifica la modifica della posizione del riquadro di lettura nei messaggi.</t>
+        </is>
+      </c>
+      <c r="D4" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare a Impostazioni &gt; Home.
+3. Verificare le opzioni 'A destra' e 'In basso'.
+4. Selezionare 'In basso'.
+5. Verificare il toast/cambio visivo.
+6. Scattare screenshot.
+7. Ripristinare 'A destra'.</t>
+        </is>
+      </c>
+      <c r="E4" s="51" t="inlineStr">
+        <is>
+          <t>Le opzioni del riquadro di lettura sono disponibili e selezionabili; la modifica viene applicata correttamente.</t>
+        </is>
+      </c>
+      <c r="F4" s="51" t="n"/>
+    </row>
+    <row r="5" ht="72.38095238095238" customHeight="1">
+      <c r="A5" s="82" t="n">
+        <v>57</v>
+      </c>
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>test_impostazioni_03.py
+test_regole_messaggi</t>
+        </is>
+      </c>
+      <c r="C5" s="58" t="inlineStr">
+        <is>
+          <t>Verifica l'accesso e la creazione di regole per i messaggi nelle Impostazioni.</t>
+        </is>
+      </c>
+      <c r="D5" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare direttamente a /new/settings/messages-writing/message-rules.
+3. Cliccare 'Nuova regola'.
+4. Verificare che il form (Nome regola, Condizioni, Azioni) sia visibile.
+5. Compilare il nome regola.
+6. Scattare screenshot.
+7. Eliminare la regola creata (cleanup).</t>
+        </is>
+      </c>
+      <c r="E5" s="58" t="inlineStr">
+        <is>
+          <t>La sezione Regole messaggi è accessibile e il form di creazione nuova regola si apre correttamente.</t>
+        </is>
+      </c>
+      <c r="F5" s="58" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="83" t="n">
+        <v>58</v>
+      </c>
+      <c r="B6" s="51" t="inlineStr">
+        <is>
+          <t>test_impostazioni_04.py
+test_risposta_automatica</t>
+        </is>
+      </c>
+      <c r="C6" s="51" t="inlineStr">
+        <is>
+          <t>Verifica l'accesso alla pagina 'Risposta automatica' nelle Impostazioni.</t>
+        </is>
+      </c>
+      <c r="D6" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare direttamente a /new/settings/messages-writing/automatic-reply.
+3. Verificare che l'h1 'Risposta automatica' sia visibile.
+4. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="E6" s="51" t="inlineStr">
+        <is>
+          <t>La pagina 'Risposta automatica' si carica correttamente con l'h1 atteso visibile.</t>
+        </is>
+      </c>
+      <c r="F6" s="51" t="inlineStr">
+        <is>
+          <t>Su PEL non esiste l'accordion 'Avvisi e report' presente su PEC: la pagina è raggiungibile solo via URL diretto (stesso namespace di Firme e Regole messaggi). URL individuato navigando manualmente dalla sidebar in debug.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="74.04761904761905" customHeight="1">
+      <c r="A7" s="82" t="n">
+        <v>59</v>
+      </c>
+      <c r="B7" s="58" t="inlineStr">
+        <is>
+          <t>test_impostazioni_05.py
+test_posta_indesiderata</t>
+        </is>
+      </c>
+      <c r="C7" s="58" t="inlineStr">
+        <is>
+          <t>Verifica la sezione Posta indesiderata e il blocco di un mittente.</t>
+        </is>
+      </c>
+      <c r="D7" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare a Impostazioni &gt; Account e sicurezza &gt; Posta indesiderata.
+3. Scattare screenshot.
+4. Verificare che la sezione sia caricata.
+5. Aggiungere un indirizzo email alla lista di blocco.
+6. Verificare che l'indirizzo sia nella lista.
+7. Rimuovere l'indirizzo (cleanup).</t>
+        </is>
+      </c>
+      <c r="E7" s="58" t="inlineStr">
+        <is>
+          <t>La sezione Posta indesiderata è accessibile; è possibile aggiungere e rimuovere indirizzi dalla lista di blocco.</t>
+        </is>
+      </c>
+      <c r="F7" s="58" t="n"/>
+    </row>
+    <row r="8" ht="81.9047619047619" customHeight="1">
+      <c r="A8" s="83" t="n">
+        <v>60</v>
+      </c>
+      <c r="B8" s="51" t="inlineStr">
+        <is>
+          <t>test_impostazioni_06.py
+test_impostazioni_cestino</t>
+        </is>
+      </c>
+      <c r="C8" s="51" t="inlineStr">
+        <is>
+          <t>Verifica le opzioni di configurazione del Cestino nelle Impostazioni.</t>
+        </is>
+      </c>
+      <c r="D8" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare direttamente a /new/settings/messages-writing/empty-trash.
+3. Attendere l'h1 'Cestino' visibile.
+4. Verificare la presenza di testo relativo allo svuotamento/eliminazione automatica.
+5. Verificare la presenza di almeno un'opzione di configurazione (select/radio/checkbox).
+6. Scattare screenshot.</t>
+        </is>
+      </c>
+      <c r="E8" s="51" t="inlineStr">
+        <is>
+          <t>La sezione Cestino nelle Impostazioni è accessibile e le opzioni di configurazione sono presenti.</t>
+        </is>
+      </c>
+      <c r="F8" s="51" t="inlineStr">
+        <is>
+          <t>Su PEL il link sidebar 'Cestino' è un bottone in shadow DOM che non supera il controllo di visibilità standard di Playwright: si naviga direttamente all'URL. Richiede un'attesa esplicita sull'h1 per evitare una race condition di caricamento SPA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="82" t="n">
+        <v>61</v>
+      </c>
+      <c r="B9" s="58" t="inlineStr">
+        <is>
+          <t>test_impostazioni_07.py
+test_storico_accessi</t>
+        </is>
+      </c>
+      <c r="C9" s="58" t="inlineStr">
+        <is>
+          <t>Verifica l'accesso e la visualizzazione dello storico degli accessi alla casella PEL.</t>
+        </is>
+      </c>
+      <c r="D9" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare direttamente a /new/settings/account-security/access-history.
+3. Scattare screenshot.
+4. Verificare che l'URL contenga 'access-history' o 'account-security' (assert).</t>
+        </is>
+      </c>
+      <c r="E9" s="58" t="inlineStr">
+        <is>
+          <t>La pagina Storico accessi è raggiungibile correttamente.</t>
+        </is>
+      </c>
+      <c r="F9" s="58" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="55" t="inlineStr">
+        <is>
+          <t>MODULO: ARCHIVIO – 2 Casi di Test</t>
+        </is>
+      </c>
+      <c r="B1" s="55" t="n"/>
+      <c r="C1" s="55" t="n"/>
+      <c r="D1" s="55" t="n"/>
+      <c r="E1" s="55" t="n"/>
+      <c r="F1" s="55" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="81" t="inlineStr">
+        <is>
+          <t>File / Funzione</t>
+        </is>
+      </c>
+      <c r="C2" s="81" t="inlineStr">
+        <is>
+          <t>Descrizione</t>
+        </is>
+      </c>
+      <c r="D2" s="81" t="inlineStr">
+        <is>
+          <t>Passi</t>
+        </is>
+      </c>
+      <c r="E2" s="81" t="inlineStr">
+        <is>
+          <t>Risultato Atteso</t>
+        </is>
+      </c>
+      <c r="F2" s="81" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="134.2857142857143" customHeight="1">
+      <c r="A3" s="82" t="n">
+        <v>53</v>
+      </c>
+      <c r="B3" s="58" t="inlineStr">
+        <is>
+          <t>test_archivio_01.py
+test_configurazione_archivio</t>
+        </is>
+      </c>
+      <c r="C3" s="58" t="inlineStr">
+        <is>
+          <t>Verifica la pagina di configurazione archivio: struttura, radio button e checkbox opzioni. Skip se la feature non è disponibile sull'account.</t>
+        </is>
+      </c>
+      <c r="D3" s="58" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare direttamente a /new/settings/archive.
+3. Se l'h1 'Archivio' non è visibile entro 10s, skip (feature non disponibile).
+4. Verificare h1 'Archivio' e h2 'Configurazione Archivio'.
+5. Verificare almeno 2 radio button e le checkbox opzioni (RA, RD, PEC ricevute/inviate).
+6. Selezionare 'Scegli quali messaggi archiviare' e una checkbox.
+7. Salvare e verificare il toast di conferma.
+8. Ricaricare e verificare che la selezione sia mantenuta.
+9. Scattare screenshot.
+10. Cleanup: ripristinare 'Archivia tutti' e salvare.</t>
+        </is>
+      </c>
+      <c r="E3" s="58" t="inlineStr">
+        <is>
+          <t>La pagina di configurazione Archivio mostra la struttura attesa e il salvataggio persiste dopo reload, oppure il test fa skip pulito se la feature non è presente.</t>
+        </is>
+      </c>
+      <c r="F3" s="58" t="inlineStr">
+        <is>
+          <t>Su PEL la feature Archivio non è disponibile su tutte le caselle (confermato dall'utente): il test fa skip automatico via pytest.skip in questo caso, comportamento atteso e non un bug.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="135.4761904761905" customHeight="1">
+      <c r="A4" s="83" t="n">
+        <v>54</v>
+      </c>
+      <c r="B4" s="51" t="inlineStr">
+        <is>
+          <t>test_archivio_02.py
+test_archivio_messaggio_inviato</t>
+        </is>
+      </c>
+      <c r="C4" s="51" t="inlineStr">
+        <is>
+          <t>Verifica che i messaggi inviati/ricevuti vengano archiviati secondo la configurazione impostata. Skip se la feature non è disponibile.</t>
+        </is>
+      </c>
+      <c r="D4" s="51" t="inlineStr">
+        <is>
+          <t>1. Accedere con credenziali valide.
+2. Navigare a /new/settings/archive; skip se la feature non è disponibile.
+3. Selezionare 'Archivia tutti i messaggi ricevuti o inviati' e salvare.
+4. Creare e inviare un messaggio PEL a se stessi con oggetto univoco.
+5. Attendere l'archiviazione (10s).
+6. Aprire la sezione Archivio tramite il menu waffle (9 punti) nell'header.
+7. Cercare il messaggio con l'oggetto univoco nella barra di ricerca dell'archivio.
+8. Scattare screenshot.
+9. Verificare che il messaggio sia presente (assert), con retry dopo 20s se non trovato subito.</t>
+        </is>
+      </c>
+      <c r="E4" s="51" t="inlineStr">
+        <is>
+          <t>Il messaggio inviato a se stessi compare nella sezione Archivio, oppure il test fa skip pulito se la feature non è presente.</t>
+        </is>
+      </c>
+      <c r="F4" s="51" t="inlineStr">
+        <is>
+          <t>Stesso comportamento di skip automatico del test S01 quando la feature Archivio non è attiva sull'account.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2439,7 +6244,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="63" t="inlineStr">
         <is>
-          <t>MODULO: IMPOSTAZIONI  –  2 Casi di Test</t>
+          <t>MODULO: IMPOSTAZIONI CALENDARIO – 2 Casi di Test</t>
         </is>
       </c>
     </row>

</xml_diff>